<commit_message>
Integrazione righe con ID 191, 376
ID 191, 376 relativi ai servizi/cda: VALIDAZIONE/LAB, non vengono gestiti dall’applicativo, così abbiamo integrato il documento con applicabilità valorizzata con NO e abbiamo inciato la razionale.
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#ENTERXX/it.entersrl/it.entersrl.extralab/4.15.4.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#ENTERXX/it.entersrl/it.entersrl.extralab/4.15.4.0/report-checklist.xlsx
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1447" uniqueCount="622">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1453" uniqueCount="623">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -1956,15 +1956,18 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 21" riportata nei documenti "casi di test PSS" e "CDA2_Profilo_Sanitario_Sintetico_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>LAB - TRASF</t>
-  </si>
-  <si>
     <t>VALIDAZIONE_CDA2_LAB_TRASF_CT1</t>
   </si>
   <si>
     <t xml:space="preserve">Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation", al fine di una futura pubblicazione, con esito positivo (status code 201), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
 Il Documento CDA2 Laboratorio dovrà essere composto in modo da risultare valido dal punto di vista sintattico, semantico, terminologico. I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso dalla sezione "CASO DI TEST- OK" riportata nei documenti "Caso di test - Trasfusionale" e "CDA2_Trasfusionale_OK" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.
 </t>
+  </si>
+  <si>
+    <t>Altro (specificare)</t>
+  </si>
+  <si>
+    <t>I nostri clienti non gestiscono gli esami per laboratorio trasfusionale</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_LAB_TRASF_CT2</t>
@@ -2947,9 +2950,6 @@
     <t>L’applicativo effettua controlli preventivi sul dato inserito</t>
   </si>
   <si>
-    <t>Altro (specificare)</t>
-  </si>
-  <si>
     <t>TIPO DOCUMENTO</t>
   </si>
   <si>
@@ -3014,6 +3014,9 @@
   </si>
   <si>
     <t>30,38,46,175,177,178,179,180,181,182,183,184,185,186,187,188,189,190, 469</t>
+  </si>
+  <si>
+    <t>LAB - TRASF</t>
   </si>
   <si>
     <t>191,376 più ove possibile fare riferimento agli "ID TEST CASE OK" del Tipo "LAB"</t>
@@ -6352,7 +6355,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="12" ht="10.5" hidden="1" customHeight="1">
+    <row r="12" ht="10.5" customHeight="1">
       <c r="A12" s="33">
         <v>29.0</v>
       </c>
@@ -6389,7 +6392,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="13" ht="10.5" hidden="1" customHeight="1">
+    <row r="13" ht="10.5" customHeight="1">
       <c r="A13" s="33">
         <v>30.0</v>
       </c>
@@ -6426,7 +6429,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="14" ht="10.5" hidden="1" customHeight="1">
+    <row r="14" ht="10.5" customHeight="1">
       <c r="A14" s="33">
         <v>31.0</v>
       </c>
@@ -6463,7 +6466,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="15" ht="10.5" hidden="1" customHeight="1">
+    <row r="15" ht="10.5" customHeight="1">
       <c r="A15" s="33">
         <v>32.0</v>
       </c>
@@ -6500,7 +6503,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="16" ht="10.5" hidden="1" customHeight="1">
+    <row r="16" ht="10.5" customHeight="1">
       <c r="A16" s="33">
         <v>33.0</v>
       </c>
@@ -6537,7 +6540,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="17" ht="10.5" hidden="1" customHeight="1">
+    <row r="17" ht="10.5" customHeight="1">
       <c r="A17" s="33">
         <v>34.0</v>
       </c>
@@ -6574,7 +6577,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="18" ht="10.5" hidden="1" customHeight="1">
+    <row r="18" ht="10.5" customHeight="1">
       <c r="A18" s="33">
         <v>35.0</v>
       </c>
@@ -6670,7 +6673,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="20" ht="10.5" hidden="1" customHeight="1">
+    <row r="20" ht="10.5" customHeight="1">
       <c r="A20" s="33">
         <v>37.0</v>
       </c>
@@ -6707,7 +6710,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="21" ht="10.5" hidden="1" customHeight="1">
+    <row r="21" ht="10.5" customHeight="1">
       <c r="A21" s="33">
         <v>38.0</v>
       </c>
@@ -6744,7 +6747,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="22" ht="10.5" hidden="1" customHeight="1">
+    <row r="22" ht="10.5" customHeight="1">
       <c r="A22" s="33">
         <v>39.0</v>
       </c>
@@ -6781,7 +6784,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" ht="10.5" hidden="1" customHeight="1">
+    <row r="23" ht="10.5" customHeight="1">
       <c r="A23" s="33">
         <v>40.0</v>
       </c>
@@ -6818,7 +6821,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="24" ht="10.5" hidden="1" customHeight="1">
+    <row r="24" ht="10.5" customHeight="1">
       <c r="A24" s="33">
         <v>41.0</v>
       </c>
@@ -6855,7 +6858,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="25" ht="10.5" hidden="1" customHeight="1">
+    <row r="25" ht="10.5" customHeight="1">
       <c r="A25" s="33">
         <v>42.0</v>
       </c>
@@ -6892,7 +6895,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="26" ht="10.5" hidden="1" customHeight="1">
+    <row r="26" ht="10.5" customHeight="1">
       <c r="A26" s="33">
         <v>43.0</v>
       </c>
@@ -6986,7 +6989,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="28" ht="10.5" hidden="1" customHeight="1">
+    <row r="28" ht="10.5" customHeight="1">
       <c r="A28" s="33">
         <v>45.0</v>
       </c>
@@ -7025,7 +7028,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="29" ht="10.5" hidden="1" customHeight="1">
+    <row r="29" ht="10.5" customHeight="1">
       <c r="A29" s="33">
         <v>46.0</v>
       </c>
@@ -7064,7 +7067,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="30" ht="10.5" hidden="1" customHeight="1">
+    <row r="30" ht="10.5" customHeight="1">
       <c r="A30" s="33">
         <v>47.0</v>
       </c>
@@ -7103,7 +7106,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="31" ht="10.5" hidden="1" customHeight="1">
+    <row r="31" ht="10.5" customHeight="1">
       <c r="A31" s="33">
         <v>48.0</v>
       </c>
@@ -7142,7 +7145,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="32" ht="10.5" hidden="1" customHeight="1">
+    <row r="32" ht="10.5" customHeight="1">
       <c r="A32" s="33">
         <v>49.0</v>
       </c>
@@ -7181,7 +7184,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="33" ht="10.5" hidden="1" customHeight="1">
+    <row r="33" ht="10.5" customHeight="1">
       <c r="A33" s="33">
         <v>50.0</v>
       </c>
@@ -7220,7 +7223,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="34" ht="10.5" hidden="1" customHeight="1">
+    <row r="34" ht="10.5" customHeight="1">
       <c r="A34" s="33">
         <v>51.0</v>
       </c>
@@ -7377,7 +7380,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="37" ht="10.5" customHeight="1">
+    <row r="37">
       <c r="A37" s="33">
         <v>56.0</v>
       </c>
@@ -7727,7 +7730,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="43" ht="10.5" hidden="1" customHeight="1">
+    <row r="43" ht="10.5" customHeight="1">
       <c r="A43" s="33">
         <v>64.0</v>
       </c>
@@ -7764,7 +7767,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="44" ht="10.5" hidden="1" customHeight="1">
+    <row r="44" ht="10.5" customHeight="1">
       <c r="A44" s="33">
         <v>66.0</v>
       </c>
@@ -7801,7 +7804,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="45" ht="10.5" hidden="1" customHeight="1">
+    <row r="45" ht="10.5" customHeight="1">
       <c r="A45" s="33">
         <v>67.0</v>
       </c>
@@ -7838,7 +7841,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="46" ht="10.5" hidden="1" customHeight="1">
+    <row r="46" ht="10.5" customHeight="1">
       <c r="A46" s="33">
         <v>68.0</v>
       </c>
@@ -7875,7 +7878,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="47" ht="10.5" hidden="1" customHeight="1">
+    <row r="47" ht="10.5" customHeight="1">
       <c r="A47" s="33">
         <v>69.0</v>
       </c>
@@ -7912,7 +7915,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="48" ht="10.5" hidden="1" customHeight="1">
+    <row r="48" ht="10.5" customHeight="1">
       <c r="A48" s="33">
         <v>70.0</v>
       </c>
@@ -7949,7 +7952,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="49" ht="10.5" hidden="1" customHeight="1">
+    <row r="49" ht="10.5" customHeight="1">
       <c r="A49" s="33">
         <v>71.0</v>
       </c>
@@ -7986,7 +7989,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="50" ht="10.5" hidden="1" customHeight="1">
+    <row r="50" ht="10.5" customHeight="1">
       <c r="A50" s="33">
         <v>72.0</v>
       </c>
@@ -8023,7 +8026,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="51" ht="10.5" hidden="1" customHeight="1">
+    <row r="51" ht="10.5" customHeight="1">
       <c r="A51" s="33">
         <v>73.0</v>
       </c>
@@ -8060,7 +8063,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="52" ht="10.5" hidden="1" customHeight="1">
+    <row r="52" ht="10.5" customHeight="1">
       <c r="A52" s="33">
         <v>74.0</v>
       </c>
@@ -8097,7 +8100,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="53" ht="10.5" hidden="1" customHeight="1">
+    <row r="53" ht="10.5" customHeight="1">
       <c r="A53" s="33">
         <v>76.0</v>
       </c>
@@ -8134,7 +8137,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="54" ht="10.5" hidden="1" customHeight="1">
+    <row r="54" ht="10.5" customHeight="1">
       <c r="A54" s="33">
         <v>78.0</v>
       </c>
@@ -8171,7 +8174,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="55" ht="10.5" hidden="1" customHeight="1">
+    <row r="55" ht="10.5" customHeight="1">
       <c r="A55" s="33">
         <v>79.0</v>
       </c>
@@ -8208,7 +8211,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="56" ht="10.5" hidden="1" customHeight="1">
+    <row r="56" ht="10.5" customHeight="1">
       <c r="A56" s="33">
         <v>80.0</v>
       </c>
@@ -8245,7 +8248,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="57" ht="10.5" hidden="1" customHeight="1">
+    <row r="57" ht="10.5" customHeight="1">
       <c r="A57" s="33">
         <v>81.0</v>
       </c>
@@ -8282,7 +8285,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="58" ht="10.5" hidden="1" customHeight="1">
+    <row r="58" ht="10.5" customHeight="1">
       <c r="A58" s="33">
         <v>83.0</v>
       </c>
@@ -8319,7 +8322,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="59" ht="10.5" hidden="1" customHeight="1">
+    <row r="59" ht="10.5" customHeight="1">
       <c r="A59" s="33">
         <v>84.0</v>
       </c>
@@ -8356,7 +8359,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="60" ht="10.5" hidden="1" customHeight="1">
+    <row r="60" ht="10.5" customHeight="1">
       <c r="A60" s="33">
         <v>85.0</v>
       </c>
@@ -8393,7 +8396,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="61" ht="10.5" hidden="1" customHeight="1">
+    <row r="61" ht="10.5" customHeight="1">
       <c r="A61" s="33">
         <v>86.0</v>
       </c>
@@ -8430,7 +8433,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="62" ht="10.5" hidden="1" customHeight="1">
+    <row r="62" ht="10.5" customHeight="1">
       <c r="A62" s="33">
         <v>87.0</v>
       </c>
@@ -8467,7 +8470,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="63" ht="10.5" hidden="1" customHeight="1">
+    <row r="63" ht="10.5" customHeight="1">
       <c r="A63" s="33">
         <v>88.0</v>
       </c>
@@ -8504,7 +8507,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="64" ht="10.5" hidden="1" customHeight="1">
+    <row r="64" ht="10.5" customHeight="1">
       <c r="A64" s="33">
         <v>89.0</v>
       </c>
@@ -8541,7 +8544,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="65" ht="10.5" hidden="1" customHeight="1">
+    <row r="65" ht="10.5" customHeight="1">
       <c r="A65" s="33">
         <v>90.0</v>
       </c>
@@ -8578,7 +8581,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="66" ht="10.5" hidden="1" customHeight="1">
+    <row r="66" ht="10.5" customHeight="1">
       <c r="A66" s="33">
         <v>91.0</v>
       </c>
@@ -8615,7 +8618,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="67" ht="10.5" hidden="1" customHeight="1">
+    <row r="67" ht="10.5" customHeight="1">
       <c r="A67" s="33">
         <v>92.0</v>
       </c>
@@ -8652,7 +8655,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="68" ht="10.5" hidden="1" customHeight="1">
+    <row r="68" ht="10.5" customHeight="1">
       <c r="A68" s="33">
         <v>93.0</v>
       </c>
@@ -8689,7 +8692,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="69" ht="10.5" hidden="1" customHeight="1">
+    <row r="69" ht="10.5" customHeight="1">
       <c r="A69" s="33">
         <v>95.0</v>
       </c>
@@ -8726,7 +8729,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="70" ht="10.5" hidden="1" customHeight="1">
+    <row r="70" ht="10.5" customHeight="1">
       <c r="A70" s="33">
         <v>97.0</v>
       </c>
@@ -8763,7 +8766,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="71" ht="10.5" hidden="1" customHeight="1">
+    <row r="71" ht="10.5" customHeight="1">
       <c r="A71" s="33">
         <v>98.0</v>
       </c>
@@ -8800,7 +8803,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="72" ht="10.5" hidden="1" customHeight="1">
+    <row r="72" ht="10.5" customHeight="1">
       <c r="A72" s="33">
         <v>99.0</v>
       </c>
@@ -8837,7 +8840,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="73" ht="10.5" hidden="1" customHeight="1">
+    <row r="73" ht="10.5" customHeight="1">
       <c r="A73" s="33">
         <v>100.0</v>
       </c>
@@ -8874,7 +8877,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="74" ht="10.5" hidden="1" customHeight="1">
+    <row r="74" ht="10.5" customHeight="1">
       <c r="A74" s="33">
         <v>101.0</v>
       </c>
@@ -8911,7 +8914,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="75" ht="10.5" hidden="1" customHeight="1">
+    <row r="75" ht="10.5" customHeight="1">
       <c r="A75" s="33">
         <v>102.0</v>
       </c>
@@ -8948,7 +8951,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="76" ht="10.5" hidden="1" customHeight="1">
+    <row r="76" ht="10.5" customHeight="1">
       <c r="A76" s="33">
         <v>103.0</v>
       </c>
@@ -8985,7 +8988,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="77" ht="10.5" hidden="1" customHeight="1">
+    <row r="77" ht="10.5" customHeight="1">
       <c r="A77" s="33">
         <v>104.0</v>
       </c>
@@ -9022,7 +9025,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="78" ht="10.5" hidden="1" customHeight="1">
+    <row r="78" ht="10.5" customHeight="1">
       <c r="A78" s="33">
         <v>105.0</v>
       </c>
@@ -9059,7 +9062,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="79" ht="10.5" hidden="1" customHeight="1">
+    <row r="79" ht="10.5" customHeight="1">
       <c r="A79" s="33">
         <v>106.0</v>
       </c>
@@ -9096,7 +9099,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="80" ht="10.5" hidden="1" customHeight="1">
+    <row r="80" ht="10.5" customHeight="1">
       <c r="A80" s="33">
         <v>108.0</v>
       </c>
@@ -9133,7 +9136,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="81" ht="10.5" hidden="1" customHeight="1">
+    <row r="81" ht="10.5" customHeight="1">
       <c r="A81" s="33">
         <v>110.0</v>
       </c>
@@ -9170,7 +9173,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="82" ht="10.5" hidden="1" customHeight="1">
+    <row r="82" ht="10.5" customHeight="1">
       <c r="A82" s="33">
         <v>111.0</v>
       </c>
@@ -9207,7 +9210,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="83" ht="10.5" hidden="1" customHeight="1">
+    <row r="83" ht="10.5" customHeight="1">
       <c r="A83" s="33">
         <v>112.0</v>
       </c>
@@ -9244,7 +9247,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="84" ht="10.5" hidden="1" customHeight="1">
+    <row r="84" ht="10.5" customHeight="1">
       <c r="A84" s="33">
         <v>113.0</v>
       </c>
@@ -9281,7 +9284,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="85" ht="10.5" hidden="1" customHeight="1">
+    <row r="85" ht="10.5" customHeight="1">
       <c r="A85" s="33">
         <v>114.0</v>
       </c>
@@ -9318,7 +9321,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="86" ht="10.5" hidden="1" customHeight="1">
+    <row r="86" ht="10.5" customHeight="1">
       <c r="A86" s="33">
         <v>115.0</v>
       </c>
@@ -9355,7 +9358,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="87" ht="10.5" hidden="1" customHeight="1">
+    <row r="87" ht="10.5" customHeight="1">
       <c r="A87" s="33">
         <v>116.0</v>
       </c>
@@ -9392,7 +9395,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="88" ht="10.5" hidden="1" customHeight="1">
+    <row r="88" ht="10.5" customHeight="1">
       <c r="A88" s="33">
         <v>117.0</v>
       </c>
@@ -9429,7 +9432,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="89" ht="10.5" hidden="1" customHeight="1">
+    <row r="89" ht="10.5" customHeight="1">
       <c r="A89" s="33">
         <v>118.0</v>
       </c>
@@ -9466,7 +9469,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="90" ht="10.5" hidden="1" customHeight="1">
+    <row r="90" ht="10.5" customHeight="1">
       <c r="A90" s="33">
         <v>119.0</v>
       </c>
@@ -9503,7 +9506,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="91" ht="10.5" hidden="1" customHeight="1">
+    <row r="91" ht="10.5" customHeight="1">
       <c r="A91" s="33">
         <v>120.0</v>
       </c>
@@ -9540,7 +9543,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="92" ht="10.5" hidden="1" customHeight="1">
+    <row r="92" ht="10.5" customHeight="1">
       <c r="A92" s="33">
         <v>121.0</v>
       </c>
@@ -9577,7 +9580,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="93" ht="10.5" hidden="1" customHeight="1">
+    <row r="93" ht="10.5" customHeight="1">
       <c r="A93" s="33">
         <v>123.0</v>
       </c>
@@ -9614,7 +9617,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="94" ht="10.5" hidden="1" customHeight="1">
+    <row r="94" ht="10.5" customHeight="1">
       <c r="A94" s="33">
         <v>125.0</v>
       </c>
@@ -9651,7 +9654,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="95" ht="10.5" hidden="1" customHeight="1">
+    <row r="95" ht="10.5" customHeight="1">
       <c r="A95" s="33">
         <v>126.0</v>
       </c>
@@ -9688,7 +9691,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="96" ht="10.5" hidden="1" customHeight="1">
+    <row r="96" ht="10.5" customHeight="1">
       <c r="A96" s="33">
         <v>127.0</v>
       </c>
@@ -9725,7 +9728,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="97" ht="10.5" hidden="1" customHeight="1">
+    <row r="97" ht="10.5" customHeight="1">
       <c r="A97" s="33">
         <v>128.0</v>
       </c>
@@ -9762,7 +9765,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="98" ht="10.5" hidden="1" customHeight="1">
+    <row r="98" ht="10.5" customHeight="1">
       <c r="A98" s="33">
         <v>129.0</v>
       </c>
@@ -9799,7 +9802,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="99" ht="10.5" hidden="1" customHeight="1">
+    <row r="99" ht="10.5" customHeight="1">
       <c r="A99" s="33">
         <v>130.0</v>
       </c>
@@ -9836,7 +9839,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="100" ht="10.5" hidden="1" customHeight="1">
+    <row r="100" ht="10.5" customHeight="1">
       <c r="A100" s="33">
         <v>131.0</v>
       </c>
@@ -9873,7 +9876,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="101" ht="10.5" hidden="1" customHeight="1">
+    <row r="101" ht="10.5" customHeight="1">
       <c r="A101" s="33">
         <v>132.0</v>
       </c>
@@ -9910,7 +9913,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="102" ht="10.5" hidden="1" customHeight="1">
+    <row r="102" ht="10.5" customHeight="1">
       <c r="A102" s="33">
         <v>133.0</v>
       </c>
@@ -9947,7 +9950,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="103" ht="10.5" hidden="1" customHeight="1">
+    <row r="103" ht="10.5" customHeight="1">
       <c r="A103" s="33">
         <v>134.0</v>
       </c>
@@ -9984,7 +9987,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="104" ht="10.5" hidden="1" customHeight="1">
+    <row r="104" ht="10.5" customHeight="1">
       <c r="A104" s="33">
         <v>135.0</v>
       </c>
@@ -10021,7 +10024,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="105" ht="10.5" hidden="1" customHeight="1">
+    <row r="105" ht="10.5" customHeight="1">
       <c r="A105" s="33">
         <v>136.0</v>
       </c>
@@ -10058,7 +10061,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="106" ht="10.5" hidden="1" customHeight="1">
+    <row r="106" ht="10.5" customHeight="1">
       <c r="A106" s="33">
         <v>137.0</v>
       </c>
@@ -10095,7 +10098,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="107" ht="10.5" hidden="1" customHeight="1">
+    <row r="107" ht="10.5" customHeight="1">
       <c r="A107" s="33">
         <v>138.0</v>
       </c>
@@ -10132,7 +10135,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="108" ht="10.5" hidden="1" customHeight="1">
+    <row r="108" ht="10.5" customHeight="1">
       <c r="A108" s="33">
         <v>139.0</v>
       </c>
@@ -10169,7 +10172,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="109" ht="10.5" hidden="1" customHeight="1">
+    <row r="109" ht="10.5" customHeight="1">
       <c r="A109" s="33">
         <v>140.0</v>
       </c>
@@ -10206,7 +10209,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="110" ht="10.5" hidden="1" customHeight="1">
+    <row r="110" ht="10.5" customHeight="1">
       <c r="A110" s="33">
         <v>141.0</v>
       </c>
@@ -10243,7 +10246,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="111" ht="10.5" hidden="1" customHeight="1">
+    <row r="111" ht="10.5" customHeight="1">
       <c r="A111" s="33">
         <v>142.0</v>
       </c>
@@ -10280,7 +10283,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="112" ht="10.5" hidden="1" customHeight="1">
+    <row r="112" ht="10.5" customHeight="1">
       <c r="A112" s="33">
         <v>143.0</v>
       </c>
@@ -10317,7 +10320,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="113" ht="10.5" hidden="1" customHeight="1">
+    <row r="113" ht="10.5" customHeight="1">
       <c r="A113" s="33">
         <v>144.0</v>
       </c>
@@ -10354,7 +10357,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="114" ht="10.5" hidden="1" customHeight="1">
+    <row r="114" ht="10.5" customHeight="1">
       <c r="A114" s="33">
         <v>145.0</v>
       </c>
@@ -10391,7 +10394,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="115" ht="10.5" hidden="1" customHeight="1">
+    <row r="115" ht="10.5" customHeight="1">
       <c r="A115" s="33">
         <v>146.0</v>
       </c>
@@ -10428,7 +10431,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="116" ht="10.5" hidden="1" customHeight="1">
+    <row r="116" ht="10.5" customHeight="1">
       <c r="A116" s="33">
         <v>152.0</v>
       </c>
@@ -10465,7 +10468,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="117" ht="10.5" hidden="1" customHeight="1">
+    <row r="117" ht="10.5" customHeight="1">
       <c r="A117" s="33">
         <v>154.0</v>
       </c>
@@ -10502,7 +10505,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="118" ht="10.5" hidden="1" customHeight="1">
+    <row r="118" ht="10.5" customHeight="1">
       <c r="A118" s="33">
         <v>155.0</v>
       </c>
@@ -10539,7 +10542,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="119" ht="10.5" hidden="1" customHeight="1">
+    <row r="119" ht="10.5" customHeight="1">
       <c r="A119" s="33">
         <v>156.0</v>
       </c>
@@ -10576,7 +10579,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="120" ht="10.5" hidden="1" customHeight="1">
+    <row r="120" ht="10.5" customHeight="1">
       <c r="A120" s="33">
         <v>159.0</v>
       </c>
@@ -10613,7 +10616,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="121" ht="10.5" hidden="1" customHeight="1">
+    <row r="121" ht="10.5" customHeight="1">
       <c r="A121" s="33">
         <v>160.0</v>
       </c>
@@ -10650,7 +10653,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="122" ht="10.5" hidden="1" customHeight="1">
+    <row r="122" ht="10.5" customHeight="1">
       <c r="A122" s="33">
         <v>161.0</v>
       </c>
@@ -10687,7 +10690,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="123" ht="10.5" hidden="1" customHeight="1">
+    <row r="123" ht="10.5" customHeight="1">
       <c r="A123" s="33">
         <v>162.0</v>
       </c>
@@ -10724,7 +10727,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="124" ht="10.5" hidden="1" customHeight="1">
+    <row r="124" ht="10.5" customHeight="1">
       <c r="A124" s="33">
         <v>163.0</v>
       </c>
@@ -10761,7 +10764,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="125" ht="10.5" hidden="1" customHeight="1">
+    <row r="125" ht="10.5" customHeight="1">
       <c r="A125" s="33">
         <v>164.0</v>
       </c>
@@ -10798,7 +10801,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="126" ht="10.5" hidden="1" customHeight="1">
+    <row r="126" ht="10.5" customHeight="1">
       <c r="A126" s="33">
         <v>165.0</v>
       </c>
@@ -10835,7 +10838,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="127" ht="10.5" hidden="1" customHeight="1">
+    <row r="127" ht="10.5" customHeight="1">
       <c r="A127" s="33">
         <v>166.0</v>
       </c>
@@ -10872,7 +10875,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="128" ht="10.5" hidden="1" customHeight="1">
+    <row r="128" ht="10.5" customHeight="1">
       <c r="A128" s="33">
         <v>167.0</v>
       </c>
@@ -10909,7 +10912,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="129" ht="10.5" hidden="1" customHeight="1">
+    <row r="129" ht="10.5" customHeight="1">
       <c r="A129" s="33">
         <v>168.0</v>
       </c>
@@ -10946,7 +10949,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="130" ht="10.5" hidden="1" customHeight="1">
+    <row r="130" ht="10.5" customHeight="1">
       <c r="A130" s="33">
         <v>169.0</v>
       </c>
@@ -10983,7 +10986,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="131" ht="10.5" hidden="1" customHeight="1">
+    <row r="131" ht="10.5" customHeight="1">
       <c r="A131" s="33">
         <v>175.0</v>
       </c>
@@ -11020,7 +11023,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="132" ht="10.5" hidden="1" customHeight="1">
+    <row r="132" ht="10.5" customHeight="1">
       <c r="A132" s="33">
         <v>177.0</v>
       </c>
@@ -11057,7 +11060,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="133" ht="10.5" hidden="1" customHeight="1">
+    <row r="133" ht="10.5" customHeight="1">
       <c r="A133" s="33">
         <v>178.0</v>
       </c>
@@ -11094,7 +11097,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="134" ht="10.5" hidden="1" customHeight="1">
+    <row r="134" ht="10.5" customHeight="1">
       <c r="A134" s="33">
         <v>179.0</v>
       </c>
@@ -11131,7 +11134,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="135" ht="10.5" hidden="1" customHeight="1">
+    <row r="135" ht="10.5" customHeight="1">
       <c r="A135" s="33">
         <v>180.0</v>
       </c>
@@ -11168,7 +11171,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="136" ht="10.5" hidden="1" customHeight="1">
+    <row r="136" ht="10.5" customHeight="1">
       <c r="A136" s="33">
         <v>181.0</v>
       </c>
@@ -11205,7 +11208,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="137" ht="10.5" hidden="1" customHeight="1">
+    <row r="137" ht="10.5" customHeight="1">
       <c r="A137" s="33">
         <v>182.0</v>
       </c>
@@ -11242,7 +11245,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="138" ht="10.5" hidden="1" customHeight="1">
+    <row r="138" ht="10.5" customHeight="1">
       <c r="A138" s="33">
         <v>183.0</v>
       </c>
@@ -11279,7 +11282,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="139" ht="10.5" hidden="1" customHeight="1">
+    <row r="139" ht="10.5" customHeight="1">
       <c r="A139" s="33">
         <v>184.0</v>
       </c>
@@ -11316,7 +11319,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="140" ht="10.5" hidden="1" customHeight="1">
+    <row r="140" ht="10.5" customHeight="1">
       <c r="A140" s="33">
         <v>185.0</v>
       </c>
@@ -11353,7 +11356,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="141" ht="10.5" hidden="1" customHeight="1">
+    <row r="141" ht="10.5" customHeight="1">
       <c r="A141" s="33">
         <v>186.0</v>
       </c>
@@ -11390,7 +11393,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="142" ht="10.5" hidden="1" customHeight="1">
+    <row r="142" ht="10.5" customHeight="1">
       <c r="A142" s="33">
         <v>187.0</v>
       </c>
@@ -11427,7 +11430,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="143" ht="10.5" hidden="1" customHeight="1">
+    <row r="143" ht="10.5" customHeight="1">
       <c r="A143" s="33">
         <v>188.0</v>
       </c>
@@ -11464,7 +11467,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="144" ht="10.5" hidden="1" customHeight="1">
+    <row r="144" ht="10.5" customHeight="1">
       <c r="A144" s="33">
         <v>189.0</v>
       </c>
@@ -11501,7 +11504,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="145" ht="10.5" hidden="1" customHeight="1">
+    <row r="145" ht="10.5" customHeight="1">
       <c r="A145" s="33">
         <v>190.0</v>
       </c>
@@ -11538,7 +11541,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="146" hidden="1">
+    <row r="146">
       <c r="A146" s="33">
         <v>191.0</v>
       </c>
@@ -11546,21 +11549,27 @@
         <v>46</v>
       </c>
       <c r="C146" s="43" t="s">
+        <v>47</v>
+      </c>
+      <c r="D146" s="33" t="s">
         <v>366</v>
       </c>
-      <c r="D146" s="33" t="s">
+      <c r="E146" s="34" t="s">
         <v>367</v>
-      </c>
-      <c r="E146" s="34" t="s">
-        <v>368</v>
       </c>
       <c r="F146" s="36"/>
       <c r="G146" s="36"/>
       <c r="H146" s="36"/>
       <c r="I146" s="41"/>
-      <c r="J146" s="37"/>
-      <c r="K146" s="37"/>
-      <c r="L146" s="37"/>
+      <c r="J146" s="42" t="s">
+        <v>61</v>
+      </c>
+      <c r="K146" s="42" t="s">
+        <v>368</v>
+      </c>
+      <c r="L146" s="42" t="s">
+        <v>369</v>
+      </c>
       <c r="M146" s="37"/>
       <c r="N146" s="37"/>
       <c r="O146" s="37"/>
@@ -11575,7 +11584,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="147" hidden="1">
+    <row r="147">
       <c r="A147" s="33">
         <v>376.0</v>
       </c>
@@ -11583,21 +11592,27 @@
         <v>46</v>
       </c>
       <c r="C147" s="43" t="s">
-        <v>366</v>
+        <v>47</v>
       </c>
       <c r="D147" s="33" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E147" s="34" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F147" s="36"/>
       <c r="G147" s="36"/>
       <c r="H147" s="36"/>
       <c r="I147" s="41"/>
-      <c r="J147" s="37"/>
-      <c r="K147" s="37"/>
-      <c r="L147" s="37"/>
+      <c r="J147" s="42" t="s">
+        <v>61</v>
+      </c>
+      <c r="K147" s="42" t="s">
+        <v>368</v>
+      </c>
+      <c r="L147" s="42" t="s">
+        <v>369</v>
+      </c>
       <c r="M147" s="37"/>
       <c r="N147" s="37"/>
       <c r="O147" s="37"/>
@@ -11612,7 +11627,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="148" ht="10.5" hidden="1" customHeight="1">
+    <row r="148" ht="10.5" customHeight="1">
       <c r="A148" s="33">
         <v>417.0</v>
       </c>
@@ -11620,13 +11635,13 @@
         <v>46</v>
       </c>
       <c r="C148" s="40" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D148" s="33" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E148" s="34" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F148" s="36"/>
       <c r="G148" s="36"/>
@@ -11649,7 +11664,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="149" ht="10.5" hidden="1" customHeight="1">
+    <row r="149" ht="10.5" customHeight="1">
       <c r="A149" s="33">
         <v>418.0</v>
       </c>
@@ -11657,13 +11672,13 @@
         <v>46</v>
       </c>
       <c r="C149" s="40" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D149" s="33" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E149" s="34" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="F149" s="36"/>
       <c r="G149" s="36"/>
@@ -11686,7 +11701,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="150" ht="10.5" hidden="1" customHeight="1">
+    <row r="150" ht="10.5" customHeight="1">
       <c r="A150" s="33">
         <v>419.0</v>
       </c>
@@ -11694,13 +11709,13 @@
         <v>46</v>
       </c>
       <c r="C150" s="40" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D150" s="33" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E150" s="34" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F150" s="36"/>
       <c r="G150" s="36"/>
@@ -11723,7 +11738,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="151" ht="10.5" hidden="1" customHeight="1">
+    <row r="151" ht="10.5" customHeight="1">
       <c r="A151" s="33">
         <v>423.0</v>
       </c>
@@ -11731,13 +11746,13 @@
         <v>46</v>
       </c>
       <c r="C151" s="40" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D151" s="33" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E151" s="34" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="F151" s="36"/>
       <c r="G151" s="36"/>
@@ -11760,7 +11775,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="152" ht="10.5" hidden="1" customHeight="1">
+    <row r="152" ht="10.5" customHeight="1">
       <c r="A152" s="33">
         <v>424.0</v>
       </c>
@@ -11768,13 +11783,13 @@
         <v>46</v>
       </c>
       <c r="C152" s="40" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D152" s="33" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="E152" s="34" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F152" s="36"/>
       <c r="G152" s="36"/>
@@ -11797,7 +11812,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="153" ht="10.5" hidden="1" customHeight="1">
+    <row r="153" ht="10.5" customHeight="1">
       <c r="A153" s="33">
         <v>425.0</v>
       </c>
@@ -11805,13 +11820,13 @@
         <v>46</v>
       </c>
       <c r="C153" s="40" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D153" s="33" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="E153" s="34" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="F153" s="36"/>
       <c r="G153" s="36"/>
@@ -11836,7 +11851,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="154" ht="10.5" hidden="1" customHeight="1">
+    <row r="154" ht="10.5" customHeight="1">
       <c r="A154" s="33">
         <v>432.0</v>
       </c>
@@ -11844,13 +11859,13 @@
         <v>46</v>
       </c>
       <c r="C154" s="40" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D154" s="33" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E154" s="34" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F154" s="36"/>
       <c r="G154" s="36"/>
@@ -11873,7 +11888,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="155" ht="10.5" hidden="1" customHeight="1">
+    <row r="155" ht="10.5" customHeight="1">
       <c r="A155" s="33">
         <v>433.0</v>
       </c>
@@ -11881,13 +11896,13 @@
         <v>46</v>
       </c>
       <c r="C155" s="40" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D155" s="33" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="E155" s="34" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="F155" s="36"/>
       <c r="G155" s="36"/>
@@ -11910,7 +11925,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="156" ht="10.5" hidden="1" customHeight="1">
+    <row r="156" ht="10.5" customHeight="1">
       <c r="A156" s="33">
         <v>434.0</v>
       </c>
@@ -11918,13 +11933,13 @@
         <v>46</v>
       </c>
       <c r="C156" s="40" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D156" s="33" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="E156" s="34" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="F156" s="36"/>
       <c r="G156" s="36"/>
@@ -11947,7 +11962,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="157" ht="10.5" hidden="1" customHeight="1">
+    <row r="157" ht="10.5" customHeight="1">
       <c r="A157" s="33">
         <v>435.0</v>
       </c>
@@ -11955,13 +11970,13 @@
         <v>46</v>
       </c>
       <c r="C157" s="40" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D157" s="33" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="E157" s="34" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="F157" s="36"/>
       <c r="G157" s="36"/>
@@ -11984,7 +11999,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="158" ht="10.5" hidden="1" customHeight="1">
+    <row r="158" ht="10.5" customHeight="1">
       <c r="A158" s="33">
         <v>437.0</v>
       </c>
@@ -11992,13 +12007,13 @@
         <v>46</v>
       </c>
       <c r="C158" s="40" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D158" s="33" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="E158" s="34" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="F158" s="36"/>
       <c r="G158" s="36"/>
@@ -12021,7 +12036,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="159" ht="10.5" hidden="1" customHeight="1">
+    <row r="159" ht="10.5" customHeight="1">
       <c r="A159" s="33">
         <v>438.0</v>
       </c>
@@ -12029,13 +12044,13 @@
         <v>46</v>
       </c>
       <c r="C159" s="40" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D159" s="33" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="E159" s="34" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="F159" s="36"/>
       <c r="G159" s="36"/>
@@ -12058,7 +12073,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="160" ht="10.5" hidden="1" customHeight="1">
+    <row r="160" ht="10.5" customHeight="1">
       <c r="A160" s="33">
         <v>440.0</v>
       </c>
@@ -12066,13 +12081,13 @@
         <v>46</v>
       </c>
       <c r="C160" s="40" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D160" s="33" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E160" s="34" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F160" s="36"/>
       <c r="G160" s="36"/>
@@ -12095,7 +12110,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="161" ht="10.5" hidden="1" customHeight="1">
+    <row r="161" ht="10.5" customHeight="1">
       <c r="A161" s="33">
         <v>441.0</v>
       </c>
@@ -12103,13 +12118,13 @@
         <v>46</v>
       </c>
       <c r="C161" s="40" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D161" s="33" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="E161" s="34" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="F161" s="36"/>
       <c r="G161" s="36"/>
@@ -12132,7 +12147,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="162" ht="10.5" hidden="1" customHeight="1">
+    <row r="162" ht="10.5" customHeight="1">
       <c r="A162" s="33">
         <v>442.0</v>
       </c>
@@ -12140,13 +12155,13 @@
         <v>46</v>
       </c>
       <c r="C162" s="40" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D162" s="33" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="E162" s="34" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="F162" s="36"/>
       <c r="G162" s="36"/>
@@ -12169,7 +12184,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="163" ht="10.5" hidden="1" customHeight="1">
+    <row r="163" ht="10.5" customHeight="1">
       <c r="A163" s="33">
         <v>443.0</v>
       </c>
@@ -12177,13 +12192,13 @@
         <v>46</v>
       </c>
       <c r="C163" s="40" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D163" s="33" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E163" s="34" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="F163" s="36"/>
       <c r="G163" s="36"/>
@@ -12206,7 +12221,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="164" ht="10.5" hidden="1" customHeight="1">
+    <row r="164" ht="10.5" customHeight="1">
       <c r="A164" s="33">
         <v>448.0</v>
       </c>
@@ -12217,10 +12232,10 @@
         <v>72</v>
       </c>
       <c r="D164" s="33" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="E164" s="34" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="F164" s="36"/>
       <c r="G164" s="36"/>
@@ -12243,7 +12258,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="165" ht="10.5" hidden="1" customHeight="1">
+    <row r="165" ht="10.5" customHeight="1">
       <c r="A165" s="33">
         <v>449.0</v>
       </c>
@@ -12254,10 +12269,10 @@
         <v>72</v>
       </c>
       <c r="D165" s="33" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="E165" s="34" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="F165" s="36"/>
       <c r="G165" s="36"/>
@@ -12280,7 +12295,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="166" ht="10.5" hidden="1" customHeight="1">
+    <row r="166" ht="10.5" customHeight="1">
       <c r="A166" s="33">
         <v>450.0</v>
       </c>
@@ -12291,10 +12306,10 @@
         <v>63</v>
       </c>
       <c r="D166" s="33" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="E166" s="34" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="F166" s="36"/>
       <c r="G166" s="36"/>
@@ -12317,7 +12332,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="167" ht="10.5" hidden="1" customHeight="1">
+    <row r="167" ht="10.5" customHeight="1">
       <c r="A167" s="33">
         <v>451.0</v>
       </c>
@@ -12328,10 +12343,10 @@
         <v>63</v>
       </c>
       <c r="D167" s="33" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E167" s="34" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="F167" s="36"/>
       <c r="G167" s="36"/>
@@ -12365,22 +12380,22 @@
         <v>47</v>
       </c>
       <c r="D168" s="33" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="E168" s="34" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="F168" s="36">
         <v>46093.0</v>
       </c>
       <c r="G168" s="36" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="H168" s="36" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="I168" s="41" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="J168" s="37" t="s">
         <v>53</v>
@@ -12401,7 +12416,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="169" ht="14.25" hidden="1" customHeight="1">
+    <row r="169" ht="14.25" customHeight="1">
       <c r="A169" s="33">
         <v>454.0</v>
       </c>
@@ -12412,10 +12427,10 @@
         <v>81</v>
       </c>
       <c r="D169" s="33" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="E169" s="34" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="F169" s="36"/>
       <c r="G169" s="36"/>
@@ -12438,7 +12453,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="170" ht="14.25" hidden="1" customHeight="1">
+    <row r="170" ht="14.25" customHeight="1">
       <c r="A170" s="33">
         <v>455.0</v>
       </c>
@@ -12449,10 +12464,10 @@
         <v>81</v>
       </c>
       <c r="D170" s="33" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="E170" s="34" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="F170" s="36"/>
       <c r="G170" s="36"/>
@@ -12475,7 +12490,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="171" ht="14.25" hidden="1" customHeight="1">
+    <row r="171" ht="14.25" customHeight="1">
       <c r="A171" s="33">
         <v>456.0</v>
       </c>
@@ -12486,10 +12501,10 @@
         <v>78</v>
       </c>
       <c r="D171" s="33" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="E171" s="34" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="F171" s="36"/>
       <c r="G171" s="36"/>
@@ -12512,7 +12527,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="172" ht="10.5" hidden="1" customHeight="1">
+    <row r="172" ht="10.5" customHeight="1">
       <c r="A172" s="33">
         <v>457.0</v>
       </c>
@@ -12523,10 +12538,10 @@
         <v>78</v>
       </c>
       <c r="D172" s="33" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="E172" s="34" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="F172" s="36"/>
       <c r="G172" s="36"/>
@@ -12549,7 +12564,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="173" ht="10.5" hidden="1" customHeight="1">
+    <row r="173" ht="10.5" customHeight="1">
       <c r="A173" s="33">
         <v>458.0</v>
       </c>
@@ -12560,10 +12575,10 @@
         <v>75</v>
       </c>
       <c r="D173" s="33" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="E173" s="34" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F173" s="36"/>
       <c r="G173" s="36"/>
@@ -12586,7 +12601,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="174" ht="14.25" hidden="1" customHeight="1">
+    <row r="174" ht="14.25" customHeight="1">
       <c r="A174" s="33">
         <v>459.0</v>
       </c>
@@ -12597,10 +12612,10 @@
         <v>75</v>
       </c>
       <c r="D174" s="33" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="E174" s="34" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="F174" s="36"/>
       <c r="G174" s="36"/>
@@ -12623,7 +12638,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="175" ht="14.25" hidden="1" customHeight="1">
+    <row r="175" ht="14.25" customHeight="1">
       <c r="A175" s="33">
         <v>460.0</v>
       </c>
@@ -12631,13 +12646,13 @@
         <v>46</v>
       </c>
       <c r="C175" s="40" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D175" s="33" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="E175" s="34" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="F175" s="36"/>
       <c r="G175" s="36"/>
@@ -12660,7 +12675,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="176" ht="14.25" hidden="1" customHeight="1">
+    <row r="176" ht="14.25" customHeight="1">
       <c r="A176" s="33">
         <v>461.0</v>
       </c>
@@ -12671,10 +12686,10 @@
         <v>72</v>
       </c>
       <c r="D176" s="33" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="E176" s="34" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="F176" s="33"/>
       <c r="G176" s="33"/>
@@ -12697,7 +12712,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="177" ht="14.25" hidden="1" customHeight="1">
+    <row r="177" ht="14.25" customHeight="1">
       <c r="A177" s="33">
         <v>462.0</v>
       </c>
@@ -12708,10 +12723,10 @@
         <v>69</v>
       </c>
       <c r="D177" s="33" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E177" s="34" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="F177" s="33"/>
       <c r="G177" s="33"/>
@@ -12734,7 +12749,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="178" ht="14.25" hidden="1" customHeight="1">
+    <row r="178" ht="14.25" customHeight="1">
       <c r="A178" s="33">
         <v>463.0</v>
       </c>
@@ -12745,10 +12760,10 @@
         <v>81</v>
       </c>
       <c r="D178" s="33" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="E178" s="34" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="F178" s="33"/>
       <c r="G178" s="33"/>
@@ -12771,7 +12786,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="179" ht="14.25" hidden="1" customHeight="1">
+    <row r="179" ht="14.25" customHeight="1">
       <c r="A179" s="33">
         <v>464.0</v>
       </c>
@@ -12782,10 +12797,10 @@
         <v>75</v>
       </c>
       <c r="D179" s="33" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="E179" s="34" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="F179" s="33"/>
       <c r="G179" s="33"/>
@@ -12808,7 +12823,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="180" ht="14.25" hidden="1" customHeight="1">
+    <row r="180" ht="14.25" customHeight="1">
       <c r="A180" s="33">
         <v>465.0</v>
       </c>
@@ -12819,10 +12834,10 @@
         <v>78</v>
       </c>
       <c r="D180" s="33" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="E180" s="34" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="F180" s="33"/>
       <c r="G180" s="33"/>
@@ -12856,22 +12871,22 @@
         <v>47</v>
       </c>
       <c r="D181" s="33" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="E181" s="34" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="F181" s="36">
         <v>46094.0</v>
       </c>
       <c r="G181" s="33" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="H181" s="33" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="I181" s="33" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J181" s="37" t="s">
         <v>53</v>
@@ -12885,7 +12900,7 @@
         <v>53</v>
       </c>
       <c r="O181" s="33" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="P181" s="37" t="s">
         <v>53</v>
@@ -12904,7 +12919,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="182" ht="14.25" hidden="1" customHeight="1">
+    <row r="182" ht="14.25" customHeight="1">
       <c r="A182" s="33">
         <v>467.0</v>
       </c>
@@ -12915,10 +12930,10 @@
         <v>63</v>
       </c>
       <c r="D182" s="33" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E182" s="34" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="F182" s="33"/>
       <c r="G182" s="33"/>
@@ -12941,7 +12956,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="183" ht="14.25" hidden="1" customHeight="1">
+    <row r="183" ht="14.25" customHeight="1">
       <c r="A183" s="33">
         <v>468.0</v>
       </c>
@@ -12952,10 +12967,10 @@
         <v>72</v>
       </c>
       <c r="D183" s="33" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="E183" s="34" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="F183" s="33"/>
       <c r="G183" s="33"/>
@@ -12978,7 +12993,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="184" ht="14.25" hidden="1" customHeight="1">
+    <row r="184" ht="14.25" customHeight="1">
       <c r="A184" s="33">
         <v>469.0</v>
       </c>
@@ -12989,10 +13004,10 @@
         <v>66</v>
       </c>
       <c r="D184" s="33" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E184" s="34" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="F184" s="33"/>
       <c r="G184" s="33"/>
@@ -13015,7 +13030,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="185" ht="14.25" hidden="1" customHeight="1">
+    <row r="185" ht="14.25" customHeight="1">
       <c r="A185" s="33">
         <v>470.0</v>
       </c>
@@ -13023,13 +13038,13 @@
         <v>46</v>
       </c>
       <c r="C185" s="40" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D185" s="33" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E185" s="34" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="F185" s="33"/>
       <c r="G185" s="33"/>
@@ -13052,7 +13067,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="186" ht="14.25" hidden="1" customHeight="1">
+    <row r="186" ht="14.25" customHeight="1">
       <c r="A186" s="33">
         <v>471.0</v>
       </c>
@@ -13063,10 +13078,10 @@
         <v>69</v>
       </c>
       <c r="D186" s="33" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="E186" s="34" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="F186" s="36"/>
       <c r="G186" s="36"/>
@@ -13089,7 +13104,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="187" ht="14.25" hidden="1" customHeight="1">
+    <row r="187" ht="14.25" customHeight="1">
       <c r="A187" s="33">
         <v>472.0</v>
       </c>
@@ -13100,10 +13115,10 @@
         <v>69</v>
       </c>
       <c r="D187" s="33" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="E187" s="34" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="F187" s="36"/>
       <c r="G187" s="36"/>
@@ -13137,22 +13152,22 @@
         <v>47</v>
       </c>
       <c r="D188" s="40" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="E188" s="34" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="F188" s="36">
         <v>46094.0</v>
       </c>
       <c r="G188" s="36" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="H188" s="36" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="I188" s="41" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="J188" s="37" t="s">
         <v>53</v>
@@ -13164,7 +13179,7 @@
       </c>
       <c r="N188" s="37"/>
       <c r="O188" s="37" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="P188" s="37" t="s">
         <v>53</v>
@@ -13183,7 +13198,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="189" ht="14.25" hidden="1" customHeight="1">
+    <row r="189" ht="14.25" customHeight="1">
       <c r="A189" s="33">
         <v>474.0</v>
       </c>
@@ -13194,10 +13209,10 @@
         <v>69</v>
       </c>
       <c r="D189" s="33" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="E189" s="34" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="F189" s="36"/>
       <c r="G189" s="36"/>
@@ -13220,7 +13235,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="190" ht="14.25" hidden="1" customHeight="1">
+    <row r="190" ht="14.25" customHeight="1">
       <c r="A190" s="33">
         <v>475.0</v>
       </c>
@@ -13231,10 +13246,10 @@
         <v>72</v>
       </c>
       <c r="D190" s="33" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="E190" s="34" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F190" s="36"/>
       <c r="G190" s="36"/>
@@ -13257,7 +13272,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="191" ht="10.5" hidden="1" customHeight="1">
+    <row r="191" ht="10.5" customHeight="1">
       <c r="A191" s="33">
         <v>476.0</v>
       </c>
@@ -13268,10 +13283,10 @@
         <v>66</v>
       </c>
       <c r="D191" s="33" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E191" s="34" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="F191" s="36"/>
       <c r="G191" s="36"/>
@@ -13294,7 +13309,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="192" ht="10.5" hidden="1" customHeight="1">
+    <row r="192" ht="10.5" customHeight="1">
       <c r="A192" s="33">
         <v>477.0</v>
       </c>
@@ -13305,10 +13320,10 @@
         <v>66</v>
       </c>
       <c r="D192" s="33" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E192" s="34" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="F192" s="36"/>
       <c r="G192" s="36"/>
@@ -13331,7 +13346,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="193" ht="10.5" hidden="1" customHeight="1">
+    <row r="193" ht="10.5" customHeight="1">
       <c r="A193" s="33">
         <v>478.0</v>
       </c>
@@ -13342,10 +13357,10 @@
         <v>66</v>
       </c>
       <c r="D193" s="33" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="E193" s="34" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="F193" s="36"/>
       <c r="G193" s="36"/>
@@ -13368,7 +13383,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="194" ht="10.5" hidden="1" customHeight="1">
+    <row r="194" ht="10.5" customHeight="1">
       <c r="A194" s="33">
         <v>479.0</v>
       </c>
@@ -13376,13 +13391,13 @@
         <v>46</v>
       </c>
       <c r="C194" s="40" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D194" s="33" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="E194" s="34" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="F194" s="36"/>
       <c r="G194" s="36"/>
@@ -13405,7 +13420,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="195" ht="10.5" hidden="1" customHeight="1">
+    <row r="195" ht="10.5" customHeight="1">
       <c r="A195" s="33">
         <v>480.0</v>
       </c>
@@ -13413,13 +13428,13 @@
         <v>46</v>
       </c>
       <c r="C195" s="40" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D195" s="33" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="E195" s="34" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="F195" s="36"/>
       <c r="G195" s="36"/>
@@ -13442,7 +13457,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="196" ht="10.5" hidden="1" customHeight="1">
+    <row r="196" ht="10.5" customHeight="1">
       <c r="A196" s="33">
         <v>481.0</v>
       </c>
@@ -13450,13 +13465,13 @@
         <v>46</v>
       </c>
       <c r="C196" s="40" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D196" s="33" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="E196" s="34" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F196" s="36"/>
       <c r="G196" s="36"/>
@@ -13479,7 +13494,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="197" ht="10.5" hidden="1" customHeight="1">
+    <row r="197" ht="10.5" customHeight="1">
       <c r="A197" s="33">
         <v>482.0</v>
       </c>
@@ -13487,13 +13502,13 @@
         <v>46</v>
       </c>
       <c r="C197" s="40" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D197" s="33" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="E197" s="34" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="F197" s="36"/>
       <c r="G197" s="36"/>
@@ -13516,7 +13531,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="198" ht="10.5" hidden="1" customHeight="1">
+    <row r="198" ht="10.5" customHeight="1">
       <c r="A198" s="33">
         <v>483.0</v>
       </c>
@@ -13524,13 +13539,13 @@
         <v>46</v>
       </c>
       <c r="C198" s="40" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D198" s="33" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="E198" s="34" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="F198" s="36"/>
       <c r="G198" s="36"/>
@@ -13553,7 +13568,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="199" ht="10.5" hidden="1" customHeight="1">
+    <row r="199" ht="10.5" customHeight="1">
       <c r="A199" s="33">
         <v>484.0</v>
       </c>
@@ -13561,13 +13576,13 @@
         <v>46</v>
       </c>
       <c r="C199" s="40" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D199" s="33" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="E199" s="34" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="F199" s="36"/>
       <c r="G199" s="36"/>
@@ -13590,7 +13605,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="200" ht="10.5" hidden="1" customHeight="1">
+    <row r="200" ht="10.5" customHeight="1">
       <c r="A200" s="33">
         <v>485.0</v>
       </c>
@@ -13598,13 +13613,13 @@
         <v>46</v>
       </c>
       <c r="C200" s="40" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D200" s="33" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="E200" s="34" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="F200" s="36"/>
       <c r="G200" s="36"/>
@@ -13627,7 +13642,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="201" ht="10.5" hidden="1" customHeight="1">
+    <row r="201" ht="10.5" customHeight="1">
       <c r="A201" s="33">
         <v>486.0</v>
       </c>
@@ -13635,13 +13650,13 @@
         <v>46</v>
       </c>
       <c r="C201" s="40" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D201" s="33" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="E201" s="34" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="F201" s="36"/>
       <c r="G201" s="36"/>
@@ -13664,7 +13679,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="202" ht="10.5" hidden="1" customHeight="1">
+    <row r="202" ht="10.5" customHeight="1">
       <c r="A202" s="33">
         <v>487.0</v>
       </c>
@@ -13672,13 +13687,13 @@
         <v>46</v>
       </c>
       <c r="C202" s="40" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D202" s="33" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="E202" s="34" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F202" s="36"/>
       <c r="G202" s="36"/>
@@ -13701,7 +13716,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="203" ht="10.5" hidden="1" customHeight="1">
+    <row r="203" ht="10.5" customHeight="1">
       <c r="A203" s="33">
         <v>488.0</v>
       </c>
@@ -13709,13 +13724,13 @@
         <v>46</v>
       </c>
       <c r="C203" s="40" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D203" s="33" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="E203" s="34" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="F203" s="36"/>
       <c r="G203" s="36"/>
@@ -13738,7 +13753,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="204" ht="10.5" hidden="1" customHeight="1">
+    <row r="204" ht="10.5" customHeight="1">
       <c r="A204" s="33">
         <v>489.0</v>
       </c>
@@ -13746,13 +13761,13 @@
         <v>46</v>
       </c>
       <c r="C204" s="40" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D204" s="33" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="E204" s="34" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F204" s="36"/>
       <c r="G204" s="36"/>
@@ -13775,7 +13790,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="205" ht="10.5" hidden="1" customHeight="1">
+    <row r="205" ht="10.5" customHeight="1">
       <c r="A205" s="33">
         <v>490.0</v>
       </c>
@@ -13783,10 +13798,10 @@
         <v>46</v>
       </c>
       <c r="C205" s="40" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D205" s="33" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E205" s="34" t="s">
         <v>104</v>
@@ -13814,7 +13829,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="206" ht="14.25" hidden="1" customHeight="1">
+    <row r="206" ht="14.25" customHeight="1">
       <c r="A206" s="33">
         <v>491.0</v>
       </c>
@@ -13822,13 +13837,13 @@
         <v>46</v>
       </c>
       <c r="C206" s="40" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D206" s="33" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="E206" s="34" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F206" s="36"/>
       <c r="G206" s="36"/>
@@ -13851,7 +13866,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="207" ht="14.25" hidden="1" customHeight="1">
+    <row r="207" ht="14.25" customHeight="1">
       <c r="A207" s="33">
         <v>492.0</v>
       </c>
@@ -13859,13 +13874,13 @@
         <v>46</v>
       </c>
       <c r="C207" s="40" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D207" s="33" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="E207" s="34" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="F207" s="36"/>
       <c r="G207" s="36"/>
@@ -13888,7 +13903,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="208" ht="14.25" hidden="1" customHeight="1">
+    <row r="208" ht="14.25" customHeight="1">
       <c r="A208" s="33">
         <v>493.0</v>
       </c>
@@ -13896,13 +13911,13 @@
         <v>46</v>
       </c>
       <c r="C208" s="40" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D208" s="33" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="E208" s="34" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="F208" s="36"/>
       <c r="G208" s="36"/>
@@ -13925,7 +13940,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="209" ht="13.5" hidden="1" customHeight="1">
+    <row r="209" ht="13.5" customHeight="1">
       <c r="A209" s="33">
         <v>494.0</v>
       </c>
@@ -13933,13 +13948,13 @@
         <v>46</v>
       </c>
       <c r="C209" s="40" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D209" s="33" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="E209" s="34" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F209" s="36"/>
       <c r="G209" s="36"/>
@@ -13962,7 +13977,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="210" ht="14.25" hidden="1" customHeight="1">
+    <row r="210" ht="14.25" customHeight="1">
       <c r="A210" s="33">
         <v>495.0</v>
       </c>
@@ -13970,13 +13985,13 @@
         <v>46</v>
       </c>
       <c r="C210" s="40" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D210" s="33" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E210" s="34" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="F210" s="36"/>
       <c r="G210" s="36"/>
@@ -13999,7 +14014,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="211" ht="14.25" hidden="1" customHeight="1">
+    <row r="211" ht="14.25" customHeight="1">
       <c r="A211" s="33">
         <v>496.0</v>
       </c>
@@ -14007,13 +14022,13 @@
         <v>46</v>
       </c>
       <c r="C211" s="40" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D211" s="33" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E211" s="34" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="F211" s="36"/>
       <c r="G211" s="36"/>
@@ -14036,7 +14051,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="212" ht="14.25" hidden="1" customHeight="1">
+    <row r="212" ht="14.25" customHeight="1">
       <c r="A212" s="33">
         <v>497.0</v>
       </c>
@@ -14044,13 +14059,13 @@
         <v>46</v>
       </c>
       <c r="C212" s="40" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D212" s="33" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="E212" s="34" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F212" s="36"/>
       <c r="G212" s="36"/>
@@ -14073,7 +14088,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="213" ht="14.25" hidden="1" customHeight="1">
+    <row r="213" ht="14.25" customHeight="1">
       <c r="A213" s="33">
         <v>498.0</v>
       </c>
@@ -14081,13 +14096,13 @@
         <v>46</v>
       </c>
       <c r="C213" s="40" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D213" s="33" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E213" s="34" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="F213" s="36"/>
       <c r="G213" s="36"/>
@@ -14110,7 +14125,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="214" ht="14.25" hidden="1" customHeight="1">
+    <row r="214" ht="14.25" customHeight="1">
       <c r="A214" s="33">
         <v>499.0</v>
       </c>
@@ -14118,13 +14133,13 @@
         <v>46</v>
       </c>
       <c r="C214" s="40" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D214" s="33" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="E214" s="34" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="F214" s="36"/>
       <c r="G214" s="36"/>
@@ -14147,7 +14162,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="215" ht="14.25" hidden="1" customHeight="1">
+    <row r="215" ht="14.25" customHeight="1">
       <c r="A215" s="33">
         <v>500.0</v>
       </c>
@@ -14155,13 +14170,13 @@
         <v>46</v>
       </c>
       <c r="C215" s="40" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D215" s="33" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E215" s="34" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="F215" s="36"/>
       <c r="G215" s="36"/>
@@ -14184,7 +14199,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="216" ht="14.25" hidden="1" customHeight="1">
+    <row r="216" ht="14.25" customHeight="1">
       <c r="A216" s="33">
         <v>501.0</v>
       </c>
@@ -14192,13 +14207,13 @@
         <v>46</v>
       </c>
       <c r="C216" s="40" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D216" s="33" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="E216" s="34" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="F216" s="36"/>
       <c r="G216" s="36"/>
@@ -14221,7 +14236,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="217" ht="14.25" hidden="1" customHeight="1">
+    <row r="217" ht="14.25" customHeight="1">
       <c r="A217" s="33">
         <v>502.0</v>
       </c>
@@ -14229,13 +14244,13 @@
         <v>46</v>
       </c>
       <c r="C217" s="40" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D217" s="33" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E217" s="34" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="F217" s="36"/>
       <c r="G217" s="36"/>
@@ -14258,7 +14273,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="218" ht="14.25" hidden="1" customHeight="1">
+    <row r="218" ht="14.25" customHeight="1">
       <c r="A218" s="33">
         <v>503.0</v>
       </c>
@@ -14266,13 +14281,13 @@
         <v>46</v>
       </c>
       <c r="C218" s="40" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D218" s="33" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="E218" s="34" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="F218" s="36"/>
       <c r="G218" s="36"/>
@@ -14295,7 +14310,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="219" ht="14.25" hidden="1" customHeight="1">
+    <row r="219" ht="14.25" customHeight="1">
       <c r="A219" s="33">
         <v>504.0</v>
       </c>
@@ -14303,13 +14318,13 @@
         <v>46</v>
       </c>
       <c r="C219" s="40" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D219" s="33" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="E219" s="34" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="F219" s="36"/>
       <c r="G219" s="36"/>
@@ -14332,7 +14347,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="220" ht="14.25" hidden="1" customHeight="1">
+    <row r="220" ht="14.25" customHeight="1">
       <c r="A220" s="33">
         <v>505.0</v>
       </c>
@@ -14340,10 +14355,10 @@
         <v>46</v>
       </c>
       <c r="C220" s="40" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D220" s="33" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="E220" s="34" t="s">
         <v>104</v>
@@ -14371,7 +14386,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="221" ht="14.25" hidden="1" customHeight="1">
+    <row r="221" ht="14.25" customHeight="1">
       <c r="A221" s="33">
         <v>506.0</v>
       </c>
@@ -14379,13 +14394,13 @@
         <v>46</v>
       </c>
       <c r="C221" s="40" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="D221" s="33" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="E221" s="34" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="F221" s="36"/>
       <c r="G221" s="36"/>
@@ -14408,7 +14423,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="222" ht="14.25" hidden="1" customHeight="1">
+    <row r="222" ht="14.25" customHeight="1">
       <c r="A222" s="33">
         <v>507.0</v>
       </c>
@@ -14416,13 +14431,13 @@
         <v>46</v>
       </c>
       <c r="C222" s="40" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="D222" s="33" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="E222" s="34" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="F222" s="36"/>
       <c r="G222" s="36"/>
@@ -14445,7 +14460,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="223" ht="14.25" hidden="1" customHeight="1">
+    <row r="223" ht="14.25" customHeight="1">
       <c r="A223" s="33">
         <v>508.0</v>
       </c>
@@ -14453,13 +14468,13 @@
         <v>46</v>
       </c>
       <c r="C223" s="40" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="D223" s="33" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="E223" s="34" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="F223" s="36"/>
       <c r="G223" s="36"/>
@@ -14482,7 +14497,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="224" ht="14.25" hidden="1" customHeight="1">
+    <row r="224" ht="14.25" customHeight="1">
       <c r="A224" s="33">
         <v>509.0</v>
       </c>
@@ -14490,13 +14505,13 @@
         <v>46</v>
       </c>
       <c r="C224" s="40" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="D224" s="33" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="E224" s="34" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="F224" s="36"/>
       <c r="G224" s="36"/>
@@ -14519,7 +14534,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="225" ht="14.25" hidden="1" customHeight="1">
+    <row r="225" ht="14.25" customHeight="1">
       <c r="A225" s="33">
         <v>510.0</v>
       </c>
@@ -14527,13 +14542,13 @@
         <v>46</v>
       </c>
       <c r="C225" s="40" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="D225" s="33" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="E225" s="34" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="F225" s="36"/>
       <c r="G225" s="36"/>
@@ -14556,7 +14571,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="226" ht="14.25" hidden="1" customHeight="1">
+    <row r="226" ht="14.25" customHeight="1">
       <c r="A226" s="33">
         <v>511.0</v>
       </c>
@@ -14564,13 +14579,13 @@
         <v>46</v>
       </c>
       <c r="C226" s="40" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="D226" s="33" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="E226" s="34" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="F226" s="36"/>
       <c r="G226" s="36"/>
@@ -14593,7 +14608,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="227" ht="14.25" hidden="1" customHeight="1">
+    <row r="227" ht="14.25" customHeight="1">
       <c r="A227" s="33">
         <v>512.0</v>
       </c>
@@ -14601,13 +14616,13 @@
         <v>46</v>
       </c>
       <c r="C227" s="40" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="D227" s="33" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="E227" s="34" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F227" s="36"/>
       <c r="G227" s="36"/>
@@ -14630,7 +14645,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="228" ht="14.25" hidden="1" customHeight="1">
+    <row r="228" ht="14.25" customHeight="1">
       <c r="A228" s="33">
         <v>513.0</v>
       </c>
@@ -14638,13 +14653,13 @@
         <v>46</v>
       </c>
       <c r="C228" s="40" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="D228" s="33" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="E228" s="34" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="F228" s="36"/>
       <c r="G228" s="36"/>
@@ -14667,7 +14682,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="229" ht="14.25" hidden="1" customHeight="1">
+    <row r="229" ht="14.25" customHeight="1">
       <c r="A229" s="33">
         <v>514.0</v>
       </c>
@@ -14675,13 +14690,13 @@
         <v>46</v>
       </c>
       <c r="C229" s="40" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="D229" s="33" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="E229" s="34" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="F229" s="36"/>
       <c r="G229" s="36"/>
@@ -14704,7 +14719,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="230" ht="14.25" hidden="1" customHeight="1">
+    <row r="230" ht="14.25" customHeight="1">
       <c r="A230" s="33">
         <v>515.0</v>
       </c>
@@ -14712,13 +14727,13 @@
         <v>46</v>
       </c>
       <c r="C230" s="40" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="D230" s="33" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="E230" s="34" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="F230" s="36"/>
       <c r="G230" s="36"/>
@@ -14741,7 +14756,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="231" ht="14.25" hidden="1" customHeight="1">
+    <row r="231" ht="14.25" customHeight="1">
       <c r="A231" s="33">
         <v>516.0</v>
       </c>
@@ -14749,13 +14764,13 @@
         <v>46</v>
       </c>
       <c r="C231" s="40" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="D231" s="33" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="E231" s="34" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="F231" s="36"/>
       <c r="G231" s="36"/>
@@ -14778,7 +14793,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="232" ht="14.25" hidden="1" customHeight="1">
+    <row r="232" ht="14.25" customHeight="1">
       <c r="A232" s="33">
         <v>517.0</v>
       </c>
@@ -14786,13 +14801,13 @@
         <v>46</v>
       </c>
       <c r="C232" s="40" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="D232" s="33" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="E232" s="34" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="F232" s="36"/>
       <c r="G232" s="36"/>
@@ -14815,7 +14830,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="233" ht="14.25" hidden="1" customHeight="1">
+    <row r="233" ht="14.25" customHeight="1">
       <c r="A233" s="33">
         <v>518.0</v>
       </c>
@@ -14823,13 +14838,13 @@
         <v>46</v>
       </c>
       <c r="C233" s="40" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="D233" s="33" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="E233" s="34" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="F233" s="36"/>
       <c r="G233" s="36"/>
@@ -14852,7 +14867,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="234" ht="14.25" hidden="1" customHeight="1">
+    <row r="234" ht="14.25" customHeight="1">
       <c r="A234" s="33">
         <v>519.0</v>
       </c>
@@ -14860,13 +14875,13 @@
         <v>46</v>
       </c>
       <c r="C234" s="40" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="D234" s="33" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="E234" s="34" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="F234" s="36"/>
       <c r="G234" s="36"/>
@@ -14889,7 +14904,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="235" ht="14.25" hidden="1" customHeight="1">
+    <row r="235" ht="14.25" customHeight="1">
       <c r="A235" s="33">
         <v>520.0</v>
       </c>
@@ -14897,10 +14912,10 @@
         <v>46</v>
       </c>
       <c r="C235" s="40" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="D235" s="33" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="E235" s="34" t="s">
         <v>104</v>
@@ -14928,7 +14943,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="236" ht="14.25" hidden="1" customHeight="1">
+    <row r="236" ht="14.25" customHeight="1">
       <c r="A236" s="33">
         <v>521.0</v>
       </c>
@@ -14936,13 +14951,13 @@
         <v>46</v>
       </c>
       <c r="C236" s="40" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="D236" s="33" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="E236" s="34" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="F236" s="36"/>
       <c r="G236" s="36"/>
@@ -14965,7 +14980,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="237" ht="14.25" hidden="1" customHeight="1">
+    <row r="237" ht="14.25" customHeight="1">
       <c r="A237" s="33">
         <v>522.0</v>
       </c>
@@ -14973,13 +14988,13 @@
         <v>46</v>
       </c>
       <c r="C237" s="40" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="D237" s="33" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="E237" s="34" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="F237" s="36"/>
       <c r="G237" s="36"/>
@@ -15002,7 +15017,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="238" ht="14.25" hidden="1" customHeight="1">
+    <row r="238" ht="14.25" customHeight="1">
       <c r="A238" s="33">
         <v>523.0</v>
       </c>
@@ -15010,13 +15025,13 @@
         <v>46</v>
       </c>
       <c r="C238" s="40" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="D238" s="33" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="E238" s="34" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="F238" s="36"/>
       <c r="G238" s="36"/>
@@ -15039,7 +15054,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="239" ht="14.25" hidden="1" customHeight="1">
+    <row r="239" ht="14.25" customHeight="1">
       <c r="A239" s="33">
         <v>524.0</v>
       </c>
@@ -15047,13 +15062,13 @@
         <v>46</v>
       </c>
       <c r="C239" s="40" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="D239" s="33" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="E239" s="34" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="F239" s="36"/>
       <c r="G239" s="36"/>
@@ -15076,7 +15091,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="240" ht="14.25" hidden="1" customHeight="1">
+    <row r="240" ht="14.25" customHeight="1">
       <c r="A240" s="33">
         <v>525.0</v>
       </c>
@@ -15084,13 +15099,13 @@
         <v>46</v>
       </c>
       <c r="C240" s="40" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="D240" s="33" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="E240" s="34" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="F240" s="36"/>
       <c r="G240" s="36"/>
@@ -15113,7 +15128,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="241" ht="14.25" hidden="1" customHeight="1">
+    <row r="241" ht="14.25" customHeight="1">
       <c r="A241" s="33">
         <v>526.0</v>
       </c>
@@ -15121,13 +15136,13 @@
         <v>46</v>
       </c>
       <c r="C241" s="40" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="D241" s="33" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="E241" s="34" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="F241" s="36"/>
       <c r="G241" s="36"/>
@@ -15150,7 +15165,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="242" ht="14.25" hidden="1" customHeight="1">
+    <row r="242" ht="14.25" customHeight="1">
       <c r="A242" s="33">
         <v>527.0</v>
       </c>
@@ -15158,13 +15173,13 @@
         <v>46</v>
       </c>
       <c r="C242" s="40" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="D242" s="33" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="E242" s="34" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="F242" s="36"/>
       <c r="G242" s="36"/>
@@ -15187,7 +15202,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="243" ht="14.25" hidden="1" customHeight="1">
+    <row r="243" ht="14.25" customHeight="1">
       <c r="A243" s="33">
         <v>528.0</v>
       </c>
@@ -15195,13 +15210,13 @@
         <v>46</v>
       </c>
       <c r="C243" s="40" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="D243" s="33" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="E243" s="34" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="F243" s="36"/>
       <c r="G243" s="36"/>
@@ -15224,7 +15239,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="244" ht="14.25" hidden="1" customHeight="1">
+    <row r="244" ht="14.25" customHeight="1">
       <c r="A244" s="33">
         <v>529.0</v>
       </c>
@@ -15232,13 +15247,13 @@
         <v>46</v>
       </c>
       <c r="C244" s="40" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="D244" s="33" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="E244" s="34" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="F244" s="36"/>
       <c r="G244" s="36"/>
@@ -15261,7 +15276,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="245" ht="14.25" hidden="1" customHeight="1">
+    <row r="245" ht="14.25" customHeight="1">
       <c r="A245" s="33">
         <v>530.0</v>
       </c>
@@ -15269,10 +15284,10 @@
         <v>46</v>
       </c>
       <c r="C245" s="40" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="D245" s="33" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="E245" s="34" t="s">
         <v>104</v>
@@ -18277,13 +18292,7 @@
     <row r="752" ht="14.25" customHeight="1"/>
     <row r="753" ht="14.25" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="$A$9:$W$245">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="LAB"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="$A$9:$W$245"/>
   <mergeCells count="7">
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
@@ -18324,42 +18333,42 @@
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
       <c r="A1" s="44" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="44" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="44" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="44" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="44" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="44" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="44" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
       <c r="A8" s="44" t="s">
-        <v>586</v>
+        <v>368</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1"/>
@@ -19512,77 +19521,77 @@
     </row>
     <row r="10">
       <c r="A10" s="49" t="s">
-        <v>366</v>
+        <v>609</v>
       </c>
       <c r="B10" s="49" t="s">
         <v>592</v>
       </c>
       <c r="C10" s="51" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="D10" s="50" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
       <c r="A11" s="49" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B11" s="49" t="s">
         <v>592</v>
       </c>
       <c r="C11" s="50" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="D11" s="51" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="49" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B12" s="49" t="s">
         <v>592</v>
       </c>
       <c r="C12" s="50" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="D12" s="51" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="49" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="B13" s="49" t="s">
         <v>592</v>
       </c>
       <c r="C13" s="50" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="D13" s="51" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
       <c r="A14" s="49" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B14" s="49" t="s">
         <v>592</v>
       </c>
       <c r="C14" s="50" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="D14" s="51" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="49" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="B15" s="49" t="s">
         <v>592</v>
@@ -19591,7 +19600,7 @@
         <v>521.0</v>
       </c>
       <c r="D15" s="51" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1">
@@ -22580,7 +22589,7 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="52" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="B2" s="52" t="s">
         <v>53</v>
@@ -22588,7 +22597,7 @@
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="52" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="B3" s="52" t="s">
         <v>61</v>

</xml_diff>

<commit_message>
Valorizzazione Colonna S di report-checklist
Aggiornata la colonna S di report-checklist per i casi di test indicati nella Vs email:
[28,36] C007: È necessario valorizzare le seguenti colonne: F, G, H, M, N, P, Q, R, S
[53,55,56,57,59,60,61,62,466,473] C007: È necessario valorizzare le seguenti colonne: F, G, H, I, M, N, P, Q, R, S
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#ENTERXX/it.entersrl/it.entersrl.extralab/4.15.4.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#ENTERXX/it.entersrl/it.entersrl.extralab/4.15.4.0/report-checklist.xlsx
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1453" uniqueCount="623">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1462" uniqueCount="622">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -338,13 +338,13 @@
     <t>47faa973759493685d49458a2e7d3f16</t>
   </si>
   <si>
-    <t>UNKNOWN_WORKFLOW_ID</t>
-  </si>
-  <si>
     <t>Seleziona lo scopo di utilizzo prima di continuare</t>
   </si>
   <si>
     <t>NO</t>
+  </si>
+  <si>
+    <t>La form del software mostra un errore all'utente con l'indicazione di contattare l'assistenza di EnterSrl - Extralab per la risuluzione dello stesso. Risolto il problema l'utente torna sulla form e reinvia il documento.</t>
   </si>
   <si>
     <t>KO</t>
@@ -1063,9 +1063,6 @@
   </si>
   <si>
     <t>Non è stata ricevuta una risposta dal server nel tempo previsto, riprovare tra 1 minuto.</t>
-  </si>
-  <si>
-    <t>Viene visualizzato un messaggio sul software in cui si indica all'operatore che la comunicazione con i servizi del ministero non è riuscita e di riprovare dopo un periodo di tempo. Nel caso l'errore si protragga di contattare l'assistenza di Enter Srl</t>
   </si>
   <si>
     <t>VALIDAZIONE_LDO_TIMEOUT</t>
@@ -6296,7 +6293,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" ht="10.5" customHeight="1">
+    <row r="11">
       <c r="A11" s="33">
         <v>28.0</v>
       </c>
@@ -6321,9 +6318,7 @@
       <c r="H11" s="36" t="s">
         <v>58</v>
       </c>
-      <c r="I11" s="41" t="s">
-        <v>59</v>
-      </c>
+      <c r="I11" s="41"/>
       <c r="J11" s="37" t="s">
         <v>53</v>
       </c>
@@ -6336,18 +6331,20 @@
         <v>53</v>
       </c>
       <c r="O11" s="37" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="P11" s="37" t="s">
         <v>53</v>
       </c>
       <c r="Q11" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="R11" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="S11" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="R11" s="37" t="s">
-        <v>61</v>
-      </c>
-      <c r="S11" s="37"/>
       <c r="T11" s="37"/>
       <c r="U11" s="38"/>
       <c r="V11" s="39"/>
@@ -6639,9 +6636,7 @@
       <c r="H19" s="36" t="s">
         <v>87</v>
       </c>
-      <c r="I19" s="41" t="s">
-        <v>59</v>
-      </c>
+      <c r="I19" s="41"/>
       <c r="J19" s="37" t="s">
         <v>53</v>
       </c>
@@ -6660,12 +6655,14 @@
         <v>53</v>
       </c>
       <c r="Q19" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="R19" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="S19" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="R19" s="37" t="s">
-        <v>61</v>
-      </c>
-      <c r="S19" s="37"/>
       <c r="T19" s="37"/>
       <c r="U19" s="38"/>
       <c r="V19" s="39"/>
@@ -6972,13 +6969,13 @@
         <v>53</v>
       </c>
       <c r="Q27" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="R27" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="S27" s="42" t="s">
         <v>61</v>
-      </c>
-      <c r="R27" s="37" t="s">
-        <v>61</v>
-      </c>
-      <c r="S27" s="42" t="s">
-        <v>106</v>
       </c>
       <c r="T27" s="37"/>
       <c r="U27" s="38" t="s">
@@ -7000,7 +6997,7 @@
         <v>63</v>
       </c>
       <c r="D28" s="33" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E28" s="34" t="s">
         <v>104</v>
@@ -7039,7 +7036,7 @@
         <v>66</v>
       </c>
       <c r="D29" s="33" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E29" s="34" t="s">
         <v>104</v>
@@ -7078,7 +7075,7 @@
         <v>69</v>
       </c>
       <c r="D30" s="33" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E30" s="34" t="s">
         <v>104</v>
@@ -7117,7 +7114,7 @@
         <v>72</v>
       </c>
       <c r="D31" s="33" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E31" s="34" t="s">
         <v>104</v>
@@ -7156,7 +7153,7 @@
         <v>75</v>
       </c>
       <c r="D32" s="33" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E32" s="34" t="s">
         <v>104</v>
@@ -7195,7 +7192,7 @@
         <v>78</v>
       </c>
       <c r="D33" s="33" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E33" s="34" t="s">
         <v>104</v>
@@ -7234,7 +7231,7 @@
         <v>81</v>
       </c>
       <c r="D34" s="33" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E34" s="34" t="s">
         <v>104</v>
@@ -7262,7 +7259,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="35" ht="10.5" customHeight="1">
+    <row r="35">
       <c r="A35" s="33">
         <v>53.0</v>
       </c>
@@ -7273,22 +7270,22 @@
         <v>47</v>
       </c>
       <c r="D35" s="33" t="s">
+        <v>113</v>
+      </c>
+      <c r="E35" s="34" t="s">
         <v>114</v>
-      </c>
-      <c r="E35" s="34" t="s">
-        <v>115</v>
       </c>
       <c r="F35" s="36">
         <v>46093.0</v>
       </c>
       <c r="G35" s="36" t="s">
+        <v>115</v>
+      </c>
+      <c r="H35" s="36" t="s">
         <v>116</v>
       </c>
-      <c r="H35" s="36" t="s">
+      <c r="I35" s="41" t="s">
         <v>117</v>
-      </c>
-      <c r="I35" s="41" t="s">
-        <v>118</v>
       </c>
       <c r="J35" s="37" t="s">
         <v>53</v>
@@ -7302,18 +7299,20 @@
         <v>53</v>
       </c>
       <c r="O35" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="P35" s="37" t="s">
         <v>53</v>
       </c>
       <c r="Q35" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="R35" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="S35" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="R35" s="37" t="s">
-        <v>61</v>
-      </c>
-      <c r="S35" s="37"/>
       <c r="T35" s="37"/>
       <c r="U35" s="38"/>
       <c r="V35" s="39"/>
@@ -7321,7 +7320,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="36" ht="10.5" customHeight="1">
+    <row r="36">
       <c r="A36" s="33">
         <v>55.0</v>
       </c>
@@ -7332,22 +7331,22 @@
         <v>47</v>
       </c>
       <c r="D36" s="33" t="s">
+        <v>119</v>
+      </c>
+      <c r="E36" s="34" t="s">
         <v>120</v>
-      </c>
-      <c r="E36" s="34" t="s">
-        <v>121</v>
       </c>
       <c r="F36" s="36">
         <v>46093.0</v>
       </c>
       <c r="G36" s="36" t="s">
+        <v>121</v>
+      </c>
+      <c r="H36" s="36" t="s">
         <v>122</v>
       </c>
-      <c r="H36" s="36" t="s">
+      <c r="I36" s="41" t="s">
         <v>123</v>
-      </c>
-      <c r="I36" s="41" t="s">
-        <v>124</v>
       </c>
       <c r="J36" s="37" t="s">
         <v>53</v>
@@ -7361,16 +7360,16 @@
         <v>53</v>
       </c>
       <c r="O36" s="37" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="P36" s="37" t="s">
         <v>53</v>
       </c>
       <c r="Q36" s="37" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="R36" s="37" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S36" s="37"/>
       <c r="T36" s="37"/>
@@ -7391,22 +7390,22 @@
         <v>47</v>
       </c>
       <c r="D37" s="33" t="s">
+        <v>125</v>
+      </c>
+      <c r="E37" s="34" t="s">
         <v>126</v>
-      </c>
-      <c r="E37" s="34" t="s">
-        <v>127</v>
       </c>
       <c r="F37" s="36">
         <v>46093.0</v>
       </c>
       <c r="G37" s="36" t="s">
+        <v>127</v>
+      </c>
+      <c r="H37" s="36" t="s">
         <v>128</v>
       </c>
-      <c r="H37" s="36" t="s">
+      <c r="I37" s="41" t="s">
         <v>129</v>
-      </c>
-      <c r="I37" s="41" t="s">
-        <v>130</v>
       </c>
       <c r="J37" s="37" t="s">
         <v>53</v>
@@ -7420,18 +7419,20 @@
         <v>53</v>
       </c>
       <c r="O37" s="37" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="P37" s="37" t="s">
         <v>53</v>
       </c>
       <c r="Q37" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="R37" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="S37" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="R37" s="37" t="s">
-        <v>61</v>
-      </c>
-      <c r="S37" s="37"/>
       <c r="T37" s="37"/>
       <c r="U37" s="38"/>
       <c r="V37" s="39"/>
@@ -7439,7 +7440,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="38" ht="10.5" customHeight="1">
+    <row r="38">
       <c r="A38" s="33">
         <v>57.0</v>
       </c>
@@ -7450,22 +7451,22 @@
         <v>47</v>
       </c>
       <c r="D38" s="33" t="s">
+        <v>131</v>
+      </c>
+      <c r="E38" s="34" t="s">
         <v>132</v>
-      </c>
-      <c r="E38" s="34" t="s">
-        <v>133</v>
       </c>
       <c r="F38" s="36">
         <v>46093.0</v>
       </c>
       <c r="G38" s="36" t="s">
+        <v>133</v>
+      </c>
+      <c r="H38" s="36" t="s">
         <v>134</v>
       </c>
-      <c r="H38" s="36" t="s">
+      <c r="I38" s="41" t="s">
         <v>135</v>
-      </c>
-      <c r="I38" s="41" t="s">
-        <v>136</v>
       </c>
       <c r="J38" s="37" t="s">
         <v>53</v>
@@ -7479,18 +7480,20 @@
         <v>53</v>
       </c>
       <c r="O38" s="37" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P38" s="37" t="s">
         <v>53</v>
       </c>
       <c r="Q38" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="R38" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="S38" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="R38" s="37" t="s">
-        <v>61</v>
-      </c>
-      <c r="S38" s="37"/>
       <c r="T38" s="37"/>
       <c r="U38" s="38"/>
       <c r="V38" s="39"/>
@@ -7498,7 +7501,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="39" ht="10.5" customHeight="1">
+    <row r="39">
       <c r="A39" s="33">
         <v>59.0</v>
       </c>
@@ -7509,22 +7512,22 @@
         <v>47</v>
       </c>
       <c r="D39" s="33" t="s">
+        <v>137</v>
+      </c>
+      <c r="E39" s="34" t="s">
         <v>138</v>
-      </c>
-      <c r="E39" s="34" t="s">
-        <v>139</v>
       </c>
       <c r="F39" s="36">
         <v>46093.0</v>
       </c>
       <c r="G39" s="36" t="s">
+        <v>139</v>
+      </c>
+      <c r="H39" s="36" t="s">
         <v>140</v>
       </c>
-      <c r="H39" s="36" t="s">
+      <c r="I39" s="41" t="s">
         <v>141</v>
-      </c>
-      <c r="I39" s="41" t="s">
-        <v>142</v>
       </c>
       <c r="J39" s="37" t="s">
         <v>53</v>
@@ -7535,19 +7538,21 @@
         <v>53</v>
       </c>
       <c r="N39" s="37" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O39" s="37"/>
       <c r="P39" s="37" t="s">
         <v>53</v>
       </c>
       <c r="Q39" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="R39" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="S39" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="R39" s="37" t="s">
-        <v>61</v>
-      </c>
-      <c r="S39" s="37"/>
       <c r="T39" s="37"/>
       <c r="U39" s="38"/>
       <c r="V39" s="39"/>
@@ -7555,7 +7560,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="40" ht="10.5" customHeight="1">
+    <row r="40">
       <c r="A40" s="33">
         <v>60.0</v>
       </c>
@@ -7566,22 +7571,22 @@
         <v>47</v>
       </c>
       <c r="D40" s="33" t="s">
+        <v>142</v>
+      </c>
+      <c r="E40" s="34" t="s">
         <v>143</v>
-      </c>
-      <c r="E40" s="34" t="s">
-        <v>144</v>
       </c>
       <c r="F40" s="36">
         <v>46094.0</v>
       </c>
       <c r="G40" s="36" t="s">
+        <v>144</v>
+      </c>
+      <c r="H40" s="36" t="s">
         <v>145</v>
       </c>
-      <c r="H40" s="36" t="s">
+      <c r="I40" s="41" t="s">
         <v>146</v>
-      </c>
-      <c r="I40" s="41" t="s">
-        <v>147</v>
       </c>
       <c r="J40" s="37" t="s">
         <v>53</v>
@@ -7595,18 +7600,20 @@
         <v>53</v>
       </c>
       <c r="O40" s="37" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="P40" s="37" t="s">
         <v>53</v>
       </c>
       <c r="Q40" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="R40" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="S40" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="R40" s="37" t="s">
-        <v>61</v>
-      </c>
-      <c r="S40" s="37"/>
       <c r="T40" s="37"/>
       <c r="U40" s="38"/>
       <c r="V40" s="39"/>
@@ -7614,7 +7621,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="41" ht="10.5" customHeight="1">
+    <row r="41" ht="29.25" customHeight="1">
       <c r="A41" s="33">
         <v>61.0</v>
       </c>
@@ -7625,22 +7632,22 @@
         <v>47</v>
       </c>
       <c r="D41" s="33" t="s">
+        <v>148</v>
+      </c>
+      <c r="E41" s="34" t="s">
         <v>149</v>
-      </c>
-      <c r="E41" s="34" t="s">
-        <v>150</v>
       </c>
       <c r="F41" s="36">
         <v>46094.0</v>
       </c>
       <c r="G41" s="36" t="s">
+        <v>150</v>
+      </c>
+      <c r="H41" s="36" t="s">
         <v>151</v>
       </c>
-      <c r="H41" s="36" t="s">
+      <c r="I41" s="41" t="s">
         <v>152</v>
-      </c>
-      <c r="I41" s="41" t="s">
-        <v>153</v>
       </c>
       <c r="J41" s="37" t="s">
         <v>53</v>
@@ -7654,18 +7661,20 @@
         <v>53</v>
       </c>
       <c r="O41" s="37" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="P41" s="37" t="s">
         <v>53</v>
       </c>
       <c r="Q41" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="R41" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="S41" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="R41" s="37" t="s">
-        <v>61</v>
-      </c>
-      <c r="S41" s="37"/>
       <c r="T41" s="37"/>
       <c r="U41" s="38"/>
       <c r="V41" s="39"/>
@@ -7673,7 +7682,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="42" ht="10.5" customHeight="1">
+    <row r="42">
       <c r="A42" s="33">
         <v>62.0</v>
       </c>
@@ -7684,22 +7693,22 @@
         <v>47</v>
       </c>
       <c r="D42" s="33" t="s">
+        <v>154</v>
+      </c>
+      <c r="E42" s="34" t="s">
         <v>155</v>
-      </c>
-      <c r="E42" s="34" t="s">
-        <v>156</v>
       </c>
       <c r="F42" s="36">
         <v>46094.0</v>
       </c>
       <c r="G42" s="36" t="s">
+        <v>156</v>
+      </c>
+      <c r="H42" s="36" t="s">
         <v>157</v>
       </c>
-      <c r="H42" s="36" t="s">
+      <c r="I42" s="41" t="s">
         <v>158</v>
-      </c>
-      <c r="I42" s="41" t="s">
-        <v>159</v>
       </c>
       <c r="J42" s="37" t="s">
         <v>53</v>
@@ -7710,19 +7719,21 @@
         <v>53</v>
       </c>
       <c r="N42" s="37" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O42" s="37"/>
       <c r="P42" s="37" t="s">
         <v>53</v>
       </c>
       <c r="Q42" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="R42" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="S42" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="R42" s="37" t="s">
-        <v>61</v>
-      </c>
-      <c r="S42" s="37"/>
       <c r="T42" s="37"/>
       <c r="U42" s="38"/>
       <c r="V42" s="39"/>
@@ -7741,10 +7752,10 @@
         <v>63</v>
       </c>
       <c r="D43" s="33" t="s">
+        <v>159</v>
+      </c>
+      <c r="E43" s="34" t="s">
         <v>160</v>
-      </c>
-      <c r="E43" s="34" t="s">
-        <v>161</v>
       </c>
       <c r="F43" s="36"/>
       <c r="G43" s="36"/>
@@ -7778,10 +7789,10 @@
         <v>63</v>
       </c>
       <c r="D44" s="33" t="s">
+        <v>161</v>
+      </c>
+      <c r="E44" s="34" t="s">
         <v>162</v>
-      </c>
-      <c r="E44" s="34" t="s">
-        <v>163</v>
       </c>
       <c r="F44" s="36"/>
       <c r="G44" s="36"/>
@@ -7815,10 +7826,10 @@
         <v>63</v>
       </c>
       <c r="D45" s="33" t="s">
+        <v>163</v>
+      </c>
+      <c r="E45" s="34" t="s">
         <v>164</v>
-      </c>
-      <c r="E45" s="34" t="s">
-        <v>165</v>
       </c>
       <c r="F45" s="36"/>
       <c r="G45" s="36"/>
@@ -7852,10 +7863,10 @@
         <v>63</v>
       </c>
       <c r="D46" s="33" t="s">
+        <v>165</v>
+      </c>
+      <c r="E46" s="34" t="s">
         <v>166</v>
-      </c>
-      <c r="E46" s="34" t="s">
-        <v>167</v>
       </c>
       <c r="F46" s="36"/>
       <c r="G46" s="36"/>
@@ -7889,10 +7900,10 @@
         <v>63</v>
       </c>
       <c r="D47" s="33" t="s">
+        <v>167</v>
+      </c>
+      <c r="E47" s="34" t="s">
         <v>168</v>
-      </c>
-      <c r="E47" s="34" t="s">
-        <v>169</v>
       </c>
       <c r="F47" s="36"/>
       <c r="G47" s="36"/>
@@ -7926,10 +7937,10 @@
         <v>63</v>
       </c>
       <c r="D48" s="33" t="s">
+        <v>169</v>
+      </c>
+      <c r="E48" s="34" t="s">
         <v>170</v>
-      </c>
-      <c r="E48" s="34" t="s">
-        <v>171</v>
       </c>
       <c r="F48" s="36"/>
       <c r="G48" s="36"/>
@@ -7963,10 +7974,10 @@
         <v>63</v>
       </c>
       <c r="D49" s="33" t="s">
+        <v>171</v>
+      </c>
+      <c r="E49" s="34" t="s">
         <v>172</v>
-      </c>
-      <c r="E49" s="34" t="s">
-        <v>173</v>
       </c>
       <c r="F49" s="36"/>
       <c r="G49" s="36"/>
@@ -8000,10 +8011,10 @@
         <v>63</v>
       </c>
       <c r="D50" s="33" t="s">
+        <v>173</v>
+      </c>
+      <c r="E50" s="34" t="s">
         <v>174</v>
-      </c>
-      <c r="E50" s="34" t="s">
-        <v>175</v>
       </c>
       <c r="F50" s="36"/>
       <c r="G50" s="36"/>
@@ -8037,10 +8048,10 @@
         <v>63</v>
       </c>
       <c r="D51" s="33" t="s">
+        <v>175</v>
+      </c>
+      <c r="E51" s="34" t="s">
         <v>176</v>
-      </c>
-      <c r="E51" s="34" t="s">
-        <v>177</v>
       </c>
       <c r="F51" s="36"/>
       <c r="G51" s="36"/>
@@ -8074,10 +8085,10 @@
         <v>63</v>
       </c>
       <c r="D52" s="33" t="s">
+        <v>177</v>
+      </c>
+      <c r="E52" s="34" t="s">
         <v>178</v>
-      </c>
-      <c r="E52" s="34" t="s">
-        <v>179</v>
       </c>
       <c r="F52" s="36"/>
       <c r="G52" s="36"/>
@@ -8111,10 +8122,10 @@
         <v>69</v>
       </c>
       <c r="D53" s="33" t="s">
+        <v>179</v>
+      </c>
+      <c r="E53" s="34" t="s">
         <v>180</v>
-      </c>
-      <c r="E53" s="34" t="s">
-        <v>181</v>
       </c>
       <c r="F53" s="36"/>
       <c r="G53" s="36"/>
@@ -8148,10 +8159,10 @@
         <v>69</v>
       </c>
       <c r="D54" s="33" t="s">
+        <v>181</v>
+      </c>
+      <c r="E54" s="34" t="s">
         <v>182</v>
-      </c>
-      <c r="E54" s="34" t="s">
-        <v>183</v>
       </c>
       <c r="F54" s="36"/>
       <c r="G54" s="36"/>
@@ -8185,10 +8196,10 @@
         <v>69</v>
       </c>
       <c r="D55" s="33" t="s">
+        <v>183</v>
+      </c>
+      <c r="E55" s="34" t="s">
         <v>184</v>
-      </c>
-      <c r="E55" s="34" t="s">
-        <v>185</v>
       </c>
       <c r="F55" s="36"/>
       <c r="G55" s="36"/>
@@ -8222,10 +8233,10 @@
         <v>69</v>
       </c>
       <c r="D56" s="33" t="s">
+        <v>185</v>
+      </c>
+      <c r="E56" s="34" t="s">
         <v>186</v>
-      </c>
-      <c r="E56" s="34" t="s">
-        <v>187</v>
       </c>
       <c r="F56" s="36"/>
       <c r="G56" s="36"/>
@@ -8259,10 +8270,10 @@
         <v>69</v>
       </c>
       <c r="D57" s="33" t="s">
+        <v>187</v>
+      </c>
+      <c r="E57" s="34" t="s">
         <v>188</v>
-      </c>
-      <c r="E57" s="34" t="s">
-        <v>189</v>
       </c>
       <c r="F57" s="36"/>
       <c r="G57" s="36"/>
@@ -8296,10 +8307,10 @@
         <v>69</v>
       </c>
       <c r="D58" s="33" t="s">
+        <v>189</v>
+      </c>
+      <c r="E58" s="34" t="s">
         <v>190</v>
-      </c>
-      <c r="E58" s="34" t="s">
-        <v>191</v>
       </c>
       <c r="F58" s="36"/>
       <c r="G58" s="36"/>
@@ -8333,10 +8344,10 @@
         <v>69</v>
       </c>
       <c r="D59" s="33" t="s">
+        <v>191</v>
+      </c>
+      <c r="E59" s="34" t="s">
         <v>192</v>
-      </c>
-      <c r="E59" s="34" t="s">
-        <v>193</v>
       </c>
       <c r="F59" s="36"/>
       <c r="G59" s="36"/>
@@ -8370,10 +8381,10 @@
         <v>69</v>
       </c>
       <c r="D60" s="33" t="s">
+        <v>193</v>
+      </c>
+      <c r="E60" s="34" t="s">
         <v>194</v>
-      </c>
-      <c r="E60" s="34" t="s">
-        <v>195</v>
       </c>
       <c r="F60" s="36"/>
       <c r="G60" s="36"/>
@@ -8407,10 +8418,10 @@
         <v>69</v>
       </c>
       <c r="D61" s="33" t="s">
+        <v>195</v>
+      </c>
+      <c r="E61" s="34" t="s">
         <v>196</v>
-      </c>
-      <c r="E61" s="34" t="s">
-        <v>197</v>
       </c>
       <c r="F61" s="36"/>
       <c r="G61" s="36"/>
@@ -8444,10 +8455,10 @@
         <v>69</v>
       </c>
       <c r="D62" s="33" t="s">
+        <v>197</v>
+      </c>
+      <c r="E62" s="34" t="s">
         <v>198</v>
-      </c>
-      <c r="E62" s="34" t="s">
-        <v>199</v>
       </c>
       <c r="F62" s="36"/>
       <c r="G62" s="36"/>
@@ -8481,10 +8492,10 @@
         <v>69</v>
       </c>
       <c r="D63" s="33" t="s">
+        <v>199</v>
+      </c>
+      <c r="E63" s="34" t="s">
         <v>200</v>
-      </c>
-      <c r="E63" s="34" t="s">
-        <v>201</v>
       </c>
       <c r="F63" s="36"/>
       <c r="G63" s="36"/>
@@ -8518,10 +8529,10 @@
         <v>69</v>
       </c>
       <c r="D64" s="33" t="s">
+        <v>201</v>
+      </c>
+      <c r="E64" s="34" t="s">
         <v>202</v>
-      </c>
-      <c r="E64" s="34" t="s">
-        <v>203</v>
       </c>
       <c r="F64" s="36"/>
       <c r="G64" s="36"/>
@@ -8555,10 +8566,10 @@
         <v>69</v>
       </c>
       <c r="D65" s="33" t="s">
+        <v>203</v>
+      </c>
+      <c r="E65" s="34" t="s">
         <v>204</v>
-      </c>
-      <c r="E65" s="34" t="s">
-        <v>205</v>
       </c>
       <c r="F65" s="36"/>
       <c r="G65" s="36"/>
@@ -8592,10 +8603,10 @@
         <v>69</v>
       </c>
       <c r="D66" s="33" t="s">
+        <v>205</v>
+      </c>
+      <c r="E66" s="34" t="s">
         <v>206</v>
-      </c>
-      <c r="E66" s="34" t="s">
-        <v>207</v>
       </c>
       <c r="F66" s="36"/>
       <c r="G66" s="36"/>
@@ -8629,10 +8640,10 @@
         <v>69</v>
       </c>
       <c r="D67" s="33" t="s">
+        <v>207</v>
+      </c>
+      <c r="E67" s="34" t="s">
         <v>208</v>
-      </c>
-      <c r="E67" s="34" t="s">
-        <v>209</v>
       </c>
       <c r="F67" s="36"/>
       <c r="G67" s="36"/>
@@ -8666,10 +8677,10 @@
         <v>69</v>
       </c>
       <c r="D68" s="33" t="s">
+        <v>209</v>
+      </c>
+      <c r="E68" s="34" t="s">
         <v>210</v>
-      </c>
-      <c r="E68" s="34" t="s">
-        <v>211</v>
       </c>
       <c r="F68" s="36"/>
       <c r="G68" s="36"/>
@@ -8703,10 +8714,10 @@
         <v>75</v>
       </c>
       <c r="D69" s="33" t="s">
+        <v>211</v>
+      </c>
+      <c r="E69" s="34" t="s">
         <v>212</v>
-      </c>
-      <c r="E69" s="34" t="s">
-        <v>213</v>
       </c>
       <c r="F69" s="36"/>
       <c r="G69" s="36"/>
@@ -8740,10 +8751,10 @@
         <v>75</v>
       </c>
       <c r="D70" s="33" t="s">
+        <v>213</v>
+      </c>
+      <c r="E70" s="34" t="s">
         <v>214</v>
-      </c>
-      <c r="E70" s="34" t="s">
-        <v>215</v>
       </c>
       <c r="F70" s="36"/>
       <c r="G70" s="36"/>
@@ -8777,10 +8788,10 @@
         <v>75</v>
       </c>
       <c r="D71" s="33" t="s">
+        <v>215</v>
+      </c>
+      <c r="E71" s="34" t="s">
         <v>216</v>
-      </c>
-      <c r="E71" s="34" t="s">
-        <v>217</v>
       </c>
       <c r="F71" s="36"/>
       <c r="G71" s="36"/>
@@ -8814,10 +8825,10 @@
         <v>75</v>
       </c>
       <c r="D72" s="33" t="s">
+        <v>217</v>
+      </c>
+      <c r="E72" s="34" t="s">
         <v>218</v>
-      </c>
-      <c r="E72" s="34" t="s">
-        <v>219</v>
       </c>
       <c r="F72" s="36"/>
       <c r="G72" s="36"/>
@@ -8851,10 +8862,10 @@
         <v>75</v>
       </c>
       <c r="D73" s="33" t="s">
+        <v>219</v>
+      </c>
+      <c r="E73" s="34" t="s">
         <v>220</v>
-      </c>
-      <c r="E73" s="34" t="s">
-        <v>221</v>
       </c>
       <c r="F73" s="36"/>
       <c r="G73" s="36"/>
@@ -8888,10 +8899,10 @@
         <v>75</v>
       </c>
       <c r="D74" s="33" t="s">
+        <v>221</v>
+      </c>
+      <c r="E74" s="34" t="s">
         <v>222</v>
-      </c>
-      <c r="E74" s="34" t="s">
-        <v>223</v>
       </c>
       <c r="F74" s="36"/>
       <c r="G74" s="36"/>
@@ -8925,10 +8936,10 @@
         <v>75</v>
       </c>
       <c r="D75" s="33" t="s">
+        <v>223</v>
+      </c>
+      <c r="E75" s="34" t="s">
         <v>224</v>
-      </c>
-      <c r="E75" s="34" t="s">
-        <v>225</v>
       </c>
       <c r="F75" s="36"/>
       <c r="G75" s="36"/>
@@ -8962,10 +8973,10 @@
         <v>75</v>
       </c>
       <c r="D76" s="33" t="s">
+        <v>225</v>
+      </c>
+      <c r="E76" s="34" t="s">
         <v>226</v>
-      </c>
-      <c r="E76" s="34" t="s">
-        <v>227</v>
       </c>
       <c r="F76" s="36"/>
       <c r="G76" s="36"/>
@@ -8999,10 +9010,10 @@
         <v>75</v>
       </c>
       <c r="D77" s="33" t="s">
+        <v>227</v>
+      </c>
+      <c r="E77" s="34" t="s">
         <v>228</v>
-      </c>
-      <c r="E77" s="34" t="s">
-        <v>229</v>
       </c>
       <c r="F77" s="36"/>
       <c r="G77" s="36"/>
@@ -9036,10 +9047,10 @@
         <v>75</v>
       </c>
       <c r="D78" s="33" t="s">
+        <v>229</v>
+      </c>
+      <c r="E78" s="34" t="s">
         <v>230</v>
-      </c>
-      <c r="E78" s="34" t="s">
-        <v>231</v>
       </c>
       <c r="F78" s="36"/>
       <c r="G78" s="36"/>
@@ -9073,10 +9084,10 @@
         <v>75</v>
       </c>
       <c r="D79" s="33" t="s">
+        <v>231</v>
+      </c>
+      <c r="E79" s="34" t="s">
         <v>232</v>
-      </c>
-      <c r="E79" s="34" t="s">
-        <v>233</v>
       </c>
       <c r="F79" s="36"/>
       <c r="G79" s="36"/>
@@ -9110,10 +9121,10 @@
         <v>78</v>
       </c>
       <c r="D80" s="33" t="s">
+        <v>233</v>
+      </c>
+      <c r="E80" s="34" t="s">
         <v>234</v>
-      </c>
-      <c r="E80" s="34" t="s">
-        <v>235</v>
       </c>
       <c r="F80" s="36"/>
       <c r="G80" s="36"/>
@@ -9147,10 +9158,10 @@
         <v>78</v>
       </c>
       <c r="D81" s="33" t="s">
+        <v>235</v>
+      </c>
+      <c r="E81" s="34" t="s">
         <v>236</v>
-      </c>
-      <c r="E81" s="34" t="s">
-        <v>237</v>
       </c>
       <c r="F81" s="36"/>
       <c r="G81" s="36"/>
@@ -9184,10 +9195,10 @@
         <v>78</v>
       </c>
       <c r="D82" s="33" t="s">
+        <v>237</v>
+      </c>
+      <c r="E82" s="34" t="s">
         <v>238</v>
-      </c>
-      <c r="E82" s="34" t="s">
-        <v>239</v>
       </c>
       <c r="F82" s="36"/>
       <c r="G82" s="36"/>
@@ -9221,10 +9232,10 @@
         <v>78</v>
       </c>
       <c r="D83" s="33" t="s">
+        <v>239</v>
+      </c>
+      <c r="E83" s="34" t="s">
         <v>240</v>
-      </c>
-      <c r="E83" s="34" t="s">
-        <v>241</v>
       </c>
       <c r="F83" s="36"/>
       <c r="G83" s="36"/>
@@ -9258,10 +9269,10 @@
         <v>78</v>
       </c>
       <c r="D84" s="33" t="s">
+        <v>241</v>
+      </c>
+      <c r="E84" s="34" t="s">
         <v>242</v>
-      </c>
-      <c r="E84" s="34" t="s">
-        <v>243</v>
       </c>
       <c r="F84" s="36"/>
       <c r="G84" s="36"/>
@@ -9295,10 +9306,10 @@
         <v>78</v>
       </c>
       <c r="D85" s="33" t="s">
+        <v>243</v>
+      </c>
+      <c r="E85" s="34" t="s">
         <v>244</v>
-      </c>
-      <c r="E85" s="34" t="s">
-        <v>245</v>
       </c>
       <c r="F85" s="36"/>
       <c r="G85" s="36"/>
@@ -9332,10 +9343,10 @@
         <v>78</v>
       </c>
       <c r="D86" s="33" t="s">
+        <v>245</v>
+      </c>
+      <c r="E86" s="34" t="s">
         <v>246</v>
-      </c>
-      <c r="E86" s="34" t="s">
-        <v>247</v>
       </c>
       <c r="F86" s="36"/>
       <c r="G86" s="36"/>
@@ -9369,10 +9380,10 @@
         <v>78</v>
       </c>
       <c r="D87" s="33" t="s">
+        <v>247</v>
+      </c>
+      <c r="E87" s="34" t="s">
         <v>248</v>
-      </c>
-      <c r="E87" s="34" t="s">
-        <v>249</v>
       </c>
       <c r="F87" s="36"/>
       <c r="G87" s="36"/>
@@ -9406,10 +9417,10 @@
         <v>78</v>
       </c>
       <c r="D88" s="33" t="s">
+        <v>249</v>
+      </c>
+      <c r="E88" s="34" t="s">
         <v>250</v>
-      </c>
-      <c r="E88" s="34" t="s">
-        <v>251</v>
       </c>
       <c r="F88" s="36"/>
       <c r="G88" s="36"/>
@@ -9443,10 +9454,10 @@
         <v>78</v>
       </c>
       <c r="D89" s="33" t="s">
+        <v>251</v>
+      </c>
+      <c r="E89" s="34" t="s">
         <v>252</v>
-      </c>
-      <c r="E89" s="34" t="s">
-        <v>253</v>
       </c>
       <c r="F89" s="36"/>
       <c r="G89" s="36"/>
@@ -9480,10 +9491,10 @@
         <v>78</v>
       </c>
       <c r="D90" s="33" t="s">
+        <v>253</v>
+      </c>
+      <c r="E90" s="34" t="s">
         <v>254</v>
-      </c>
-      <c r="E90" s="34" t="s">
-        <v>255</v>
       </c>
       <c r="F90" s="36"/>
       <c r="G90" s="36"/>
@@ -9517,10 +9528,10 @@
         <v>78</v>
       </c>
       <c r="D91" s="33" t="s">
+        <v>255</v>
+      </c>
+      <c r="E91" s="34" t="s">
         <v>256</v>
-      </c>
-      <c r="E91" s="34" t="s">
-        <v>257</v>
       </c>
       <c r="F91" s="36"/>
       <c r="G91" s="36"/>
@@ -9554,10 +9565,10 @@
         <v>78</v>
       </c>
       <c r="D92" s="33" t="s">
+        <v>257</v>
+      </c>
+      <c r="E92" s="34" t="s">
         <v>258</v>
-      </c>
-      <c r="E92" s="34" t="s">
-        <v>259</v>
       </c>
       <c r="F92" s="36"/>
       <c r="G92" s="36"/>
@@ -9591,10 +9602,10 @@
         <v>81</v>
       </c>
       <c r="D93" s="33" t="s">
+        <v>259</v>
+      </c>
+      <c r="E93" s="34" t="s">
         <v>260</v>
-      </c>
-      <c r="E93" s="34" t="s">
-        <v>261</v>
       </c>
       <c r="F93" s="36"/>
       <c r="G93" s="36"/>
@@ -9628,10 +9639,10 @@
         <v>81</v>
       </c>
       <c r="D94" s="33" t="s">
+        <v>261</v>
+      </c>
+      <c r="E94" s="34" t="s">
         <v>262</v>
-      </c>
-      <c r="E94" s="34" t="s">
-        <v>263</v>
       </c>
       <c r="F94" s="36"/>
       <c r="G94" s="36"/>
@@ -9665,10 +9676,10 @@
         <v>81</v>
       </c>
       <c r="D95" s="33" t="s">
+        <v>263</v>
+      </c>
+      <c r="E95" s="34" t="s">
         <v>264</v>
-      </c>
-      <c r="E95" s="34" t="s">
-        <v>265</v>
       </c>
       <c r="F95" s="36"/>
       <c r="G95" s="36"/>
@@ -9702,10 +9713,10 @@
         <v>81</v>
       </c>
       <c r="D96" s="33" t="s">
+        <v>265</v>
+      </c>
+      <c r="E96" s="34" t="s">
         <v>266</v>
-      </c>
-      <c r="E96" s="34" t="s">
-        <v>267</v>
       </c>
       <c r="F96" s="36"/>
       <c r="G96" s="36"/>
@@ -9739,10 +9750,10 @@
         <v>81</v>
       </c>
       <c r="D97" s="33" t="s">
+        <v>267</v>
+      </c>
+      <c r="E97" s="34" t="s">
         <v>268</v>
-      </c>
-      <c r="E97" s="34" t="s">
-        <v>269</v>
       </c>
       <c r="F97" s="36"/>
       <c r="G97" s="36"/>
@@ -9776,10 +9787,10 @@
         <v>81</v>
       </c>
       <c r="D98" s="33" t="s">
+        <v>269</v>
+      </c>
+      <c r="E98" s="34" t="s">
         <v>270</v>
-      </c>
-      <c r="E98" s="34" t="s">
-        <v>271</v>
       </c>
       <c r="F98" s="36"/>
       <c r="G98" s="36"/>
@@ -9813,10 +9824,10 @@
         <v>81</v>
       </c>
       <c r="D99" s="33" t="s">
+        <v>271</v>
+      </c>
+      <c r="E99" s="34" t="s">
         <v>272</v>
-      </c>
-      <c r="E99" s="34" t="s">
-        <v>273</v>
       </c>
       <c r="F99" s="36"/>
       <c r="G99" s="36"/>
@@ -9850,10 +9861,10 @@
         <v>81</v>
       </c>
       <c r="D100" s="33" t="s">
+        <v>273</v>
+      </c>
+      <c r="E100" s="34" t="s">
         <v>274</v>
-      </c>
-      <c r="E100" s="34" t="s">
-        <v>275</v>
       </c>
       <c r="F100" s="36"/>
       <c r="G100" s="36"/>
@@ -9887,10 +9898,10 @@
         <v>81</v>
       </c>
       <c r="D101" s="33" t="s">
+        <v>275</v>
+      </c>
+      <c r="E101" s="34" t="s">
         <v>276</v>
-      </c>
-      <c r="E101" s="34" t="s">
-        <v>277</v>
       </c>
       <c r="F101" s="36"/>
       <c r="G101" s="36"/>
@@ -9924,10 +9935,10 @@
         <v>81</v>
       </c>
       <c r="D102" s="33" t="s">
+        <v>277</v>
+      </c>
+      <c r="E102" s="34" t="s">
         <v>278</v>
-      </c>
-      <c r="E102" s="34" t="s">
-        <v>279</v>
       </c>
       <c r="F102" s="36"/>
       <c r="G102" s="36"/>
@@ -9961,10 +9972,10 @@
         <v>81</v>
       </c>
       <c r="D103" s="33" t="s">
+        <v>279</v>
+      </c>
+      <c r="E103" s="34" t="s">
         <v>280</v>
-      </c>
-      <c r="E103" s="34" t="s">
-        <v>281</v>
       </c>
       <c r="F103" s="36"/>
       <c r="G103" s="36"/>
@@ -9998,10 +10009,10 @@
         <v>81</v>
       </c>
       <c r="D104" s="33" t="s">
+        <v>281</v>
+      </c>
+      <c r="E104" s="34" t="s">
         <v>282</v>
-      </c>
-      <c r="E104" s="34" t="s">
-        <v>283</v>
       </c>
       <c r="F104" s="36"/>
       <c r="G104" s="36"/>
@@ -10035,10 +10046,10 @@
         <v>81</v>
       </c>
       <c r="D105" s="33" t="s">
+        <v>283</v>
+      </c>
+      <c r="E105" s="34" t="s">
         <v>284</v>
-      </c>
-      <c r="E105" s="34" t="s">
-        <v>285</v>
       </c>
       <c r="F105" s="36"/>
       <c r="G105" s="36"/>
@@ -10072,10 +10083,10 @@
         <v>81</v>
       </c>
       <c r="D106" s="33" t="s">
+        <v>285</v>
+      </c>
+      <c r="E106" s="34" t="s">
         <v>286</v>
-      </c>
-      <c r="E106" s="34" t="s">
-        <v>287</v>
       </c>
       <c r="F106" s="36"/>
       <c r="G106" s="36"/>
@@ -10109,10 +10120,10 @@
         <v>81</v>
       </c>
       <c r="D107" s="33" t="s">
+        <v>287</v>
+      </c>
+      <c r="E107" s="34" t="s">
         <v>288</v>
-      </c>
-      <c r="E107" s="34" t="s">
-        <v>289</v>
       </c>
       <c r="F107" s="36"/>
       <c r="G107" s="36"/>
@@ -10146,10 +10157,10 @@
         <v>81</v>
       </c>
       <c r="D108" s="33" t="s">
+        <v>289</v>
+      </c>
+      <c r="E108" s="34" t="s">
         <v>290</v>
-      </c>
-      <c r="E108" s="34" t="s">
-        <v>291</v>
       </c>
       <c r="F108" s="36"/>
       <c r="G108" s="36"/>
@@ -10183,10 +10194,10 @@
         <v>81</v>
       </c>
       <c r="D109" s="33" t="s">
+        <v>291</v>
+      </c>
+      <c r="E109" s="34" t="s">
         <v>292</v>
-      </c>
-      <c r="E109" s="34" t="s">
-        <v>293</v>
       </c>
       <c r="F109" s="36"/>
       <c r="G109" s="36"/>
@@ -10220,10 +10231,10 @@
         <v>81</v>
       </c>
       <c r="D110" s="33" t="s">
+        <v>293</v>
+      </c>
+      <c r="E110" s="34" t="s">
         <v>294</v>
-      </c>
-      <c r="E110" s="34" t="s">
-        <v>295</v>
       </c>
       <c r="F110" s="36"/>
       <c r="G110" s="36"/>
@@ -10257,10 +10268,10 @@
         <v>81</v>
       </c>
       <c r="D111" s="33" t="s">
+        <v>295</v>
+      </c>
+      <c r="E111" s="34" t="s">
         <v>296</v>
-      </c>
-      <c r="E111" s="34" t="s">
-        <v>297</v>
       </c>
       <c r="F111" s="36"/>
       <c r="G111" s="36"/>
@@ -10294,10 +10305,10 @@
         <v>81</v>
       </c>
       <c r="D112" s="33" t="s">
+        <v>297</v>
+      </c>
+      <c r="E112" s="34" t="s">
         <v>298</v>
-      </c>
-      <c r="E112" s="34" t="s">
-        <v>299</v>
       </c>
       <c r="F112" s="36"/>
       <c r="G112" s="36"/>
@@ -10331,10 +10342,10 @@
         <v>81</v>
       </c>
       <c r="D113" s="33" t="s">
+        <v>299</v>
+      </c>
+      <c r="E113" s="34" t="s">
         <v>300</v>
-      </c>
-      <c r="E113" s="34" t="s">
-        <v>301</v>
       </c>
       <c r="F113" s="36"/>
       <c r="G113" s="36"/>
@@ -10368,10 +10379,10 @@
         <v>81</v>
       </c>
       <c r="D114" s="33" t="s">
+        <v>301</v>
+      </c>
+      <c r="E114" s="34" t="s">
         <v>302</v>
-      </c>
-      <c r="E114" s="34" t="s">
-        <v>303</v>
       </c>
       <c r="F114" s="36"/>
       <c r="G114" s="36"/>
@@ -10405,10 +10416,10 @@
         <v>81</v>
       </c>
       <c r="D115" s="33" t="s">
+        <v>303</v>
+      </c>
+      <c r="E115" s="34" t="s">
         <v>304</v>
-      </c>
-      <c r="E115" s="34" t="s">
-        <v>305</v>
       </c>
       <c r="F115" s="36"/>
       <c r="G115" s="36"/>
@@ -10442,10 +10453,10 @@
         <v>72</v>
       </c>
       <c r="D116" s="33" t="s">
+        <v>305</v>
+      </c>
+      <c r="E116" s="34" t="s">
         <v>306</v>
-      </c>
-      <c r="E116" s="34" t="s">
-        <v>307</v>
       </c>
       <c r="F116" s="36"/>
       <c r="G116" s="36"/>
@@ -10479,10 +10490,10 @@
         <v>72</v>
       </c>
       <c r="D117" s="33" t="s">
+        <v>307</v>
+      </c>
+      <c r="E117" s="34" t="s">
         <v>308</v>
-      </c>
-      <c r="E117" s="34" t="s">
-        <v>309</v>
       </c>
       <c r="F117" s="36"/>
       <c r="G117" s="36"/>
@@ -10516,10 +10527,10 @@
         <v>72</v>
       </c>
       <c r="D118" s="33" t="s">
+        <v>309</v>
+      </c>
+      <c r="E118" s="34" t="s">
         <v>310</v>
-      </c>
-      <c r="E118" s="34" t="s">
-        <v>311</v>
       </c>
       <c r="F118" s="36"/>
       <c r="G118" s="36"/>
@@ -10553,10 +10564,10 @@
         <v>72</v>
       </c>
       <c r="D119" s="33" t="s">
+        <v>311</v>
+      </c>
+      <c r="E119" s="34" t="s">
         <v>312</v>
-      </c>
-      <c r="E119" s="34" t="s">
-        <v>313</v>
       </c>
       <c r="F119" s="36"/>
       <c r="G119" s="36"/>
@@ -10590,10 +10601,10 @@
         <v>72</v>
       </c>
       <c r="D120" s="33" t="s">
+        <v>313</v>
+      </c>
+      <c r="E120" s="34" t="s">
         <v>314</v>
-      </c>
-      <c r="E120" s="34" t="s">
-        <v>315</v>
       </c>
       <c r="F120" s="36"/>
       <c r="G120" s="36"/>
@@ -10627,10 +10638,10 @@
         <v>72</v>
       </c>
       <c r="D121" s="33" t="s">
+        <v>315</v>
+      </c>
+      <c r="E121" s="34" t="s">
         <v>316</v>
-      </c>
-      <c r="E121" s="34" t="s">
-        <v>317</v>
       </c>
       <c r="F121" s="36"/>
       <c r="G121" s="36"/>
@@ -10664,10 +10675,10 @@
         <v>72</v>
       </c>
       <c r="D122" s="33" t="s">
+        <v>317</v>
+      </c>
+      <c r="E122" s="34" t="s">
         <v>318</v>
-      </c>
-      <c r="E122" s="34" t="s">
-        <v>319</v>
       </c>
       <c r="F122" s="36"/>
       <c r="G122" s="36"/>
@@ -10701,10 +10712,10 @@
         <v>72</v>
       </c>
       <c r="D123" s="33" t="s">
+        <v>319</v>
+      </c>
+      <c r="E123" s="34" t="s">
         <v>320</v>
-      </c>
-      <c r="E123" s="34" t="s">
-        <v>321</v>
       </c>
       <c r="F123" s="36"/>
       <c r="G123" s="36"/>
@@ -10738,10 +10749,10 @@
         <v>72</v>
       </c>
       <c r="D124" s="33" t="s">
+        <v>321</v>
+      </c>
+      <c r="E124" s="34" t="s">
         <v>322</v>
-      </c>
-      <c r="E124" s="34" t="s">
-        <v>323</v>
       </c>
       <c r="F124" s="36"/>
       <c r="G124" s="36"/>
@@ -10775,10 +10786,10 @@
         <v>72</v>
       </c>
       <c r="D125" s="33" t="s">
+        <v>323</v>
+      </c>
+      <c r="E125" s="34" t="s">
         <v>324</v>
-      </c>
-      <c r="E125" s="34" t="s">
-        <v>325</v>
       </c>
       <c r="F125" s="36"/>
       <c r="G125" s="36"/>
@@ -10812,10 +10823,10 @@
         <v>72</v>
       </c>
       <c r="D126" s="33" t="s">
+        <v>325</v>
+      </c>
+      <c r="E126" s="34" t="s">
         <v>326</v>
-      </c>
-      <c r="E126" s="34" t="s">
-        <v>327</v>
       </c>
       <c r="F126" s="36"/>
       <c r="G126" s="36"/>
@@ -10849,10 +10860,10 @@
         <v>72</v>
       </c>
       <c r="D127" s="33" t="s">
+        <v>327</v>
+      </c>
+      <c r="E127" s="34" t="s">
         <v>328</v>
-      </c>
-      <c r="E127" s="34" t="s">
-        <v>329</v>
       </c>
       <c r="F127" s="36"/>
       <c r="G127" s="36"/>
@@ -10886,10 +10897,10 @@
         <v>72</v>
       </c>
       <c r="D128" s="33" t="s">
+        <v>329</v>
+      </c>
+      <c r="E128" s="34" t="s">
         <v>330</v>
-      </c>
-      <c r="E128" s="34" t="s">
-        <v>331</v>
       </c>
       <c r="F128" s="36"/>
       <c r="G128" s="36"/>
@@ -10923,10 +10934,10 @@
         <v>72</v>
       </c>
       <c r="D129" s="33" t="s">
+        <v>331</v>
+      </c>
+      <c r="E129" s="34" t="s">
         <v>332</v>
-      </c>
-      <c r="E129" s="34" t="s">
-        <v>333</v>
       </c>
       <c r="F129" s="36"/>
       <c r="G129" s="36"/>
@@ -10960,10 +10971,10 @@
         <v>72</v>
       </c>
       <c r="D130" s="33" t="s">
+        <v>333</v>
+      </c>
+      <c r="E130" s="34" t="s">
         <v>334</v>
-      </c>
-      <c r="E130" s="34" t="s">
-        <v>335</v>
       </c>
       <c r="F130" s="36"/>
       <c r="G130" s="36"/>
@@ -10997,10 +11008,10 @@
         <v>66</v>
       </c>
       <c r="D131" s="33" t="s">
+        <v>335</v>
+      </c>
+      <c r="E131" s="34" t="s">
         <v>336</v>
-      </c>
-      <c r="E131" s="34" t="s">
-        <v>337</v>
       </c>
       <c r="F131" s="36"/>
       <c r="G131" s="36"/>
@@ -11034,10 +11045,10 @@
         <v>66</v>
       </c>
       <c r="D132" s="33" t="s">
+        <v>337</v>
+      </c>
+      <c r="E132" s="34" t="s">
         <v>338</v>
-      </c>
-      <c r="E132" s="34" t="s">
-        <v>339</v>
       </c>
       <c r="F132" s="36"/>
       <c r="G132" s="36"/>
@@ -11071,10 +11082,10 @@
         <v>66</v>
       </c>
       <c r="D133" s="33" t="s">
+        <v>339</v>
+      </c>
+      <c r="E133" s="34" t="s">
         <v>340</v>
-      </c>
-      <c r="E133" s="34" t="s">
-        <v>341</v>
       </c>
       <c r="F133" s="36"/>
       <c r="G133" s="36"/>
@@ -11108,10 +11119,10 @@
         <v>66</v>
       </c>
       <c r="D134" s="33" t="s">
+        <v>341</v>
+      </c>
+      <c r="E134" s="34" t="s">
         <v>342</v>
-      </c>
-      <c r="E134" s="34" t="s">
-        <v>343</v>
       </c>
       <c r="F134" s="36"/>
       <c r="G134" s="36"/>
@@ -11145,10 +11156,10 @@
         <v>66</v>
       </c>
       <c r="D135" s="33" t="s">
+        <v>343</v>
+      </c>
+      <c r="E135" s="34" t="s">
         <v>344</v>
-      </c>
-      <c r="E135" s="34" t="s">
-        <v>345</v>
       </c>
       <c r="F135" s="36"/>
       <c r="G135" s="36"/>
@@ -11182,10 +11193,10 @@
         <v>66</v>
       </c>
       <c r="D136" s="33" t="s">
+        <v>345</v>
+      </c>
+      <c r="E136" s="34" t="s">
         <v>346</v>
-      </c>
-      <c r="E136" s="34" t="s">
-        <v>347</v>
       </c>
       <c r="F136" s="36"/>
       <c r="G136" s="36"/>
@@ -11219,10 +11230,10 @@
         <v>66</v>
       </c>
       <c r="D137" s="33" t="s">
+        <v>347</v>
+      </c>
+      <c r="E137" s="34" t="s">
         <v>348</v>
-      </c>
-      <c r="E137" s="34" t="s">
-        <v>349</v>
       </c>
       <c r="F137" s="36"/>
       <c r="G137" s="36"/>
@@ -11256,10 +11267,10 @@
         <v>66</v>
       </c>
       <c r="D138" s="33" t="s">
+        <v>349</v>
+      </c>
+      <c r="E138" s="34" t="s">
         <v>350</v>
-      </c>
-      <c r="E138" s="34" t="s">
-        <v>351</v>
       </c>
       <c r="F138" s="36"/>
       <c r="G138" s="36"/>
@@ -11293,10 +11304,10 @@
         <v>66</v>
       </c>
       <c r="D139" s="33" t="s">
+        <v>351</v>
+      </c>
+      <c r="E139" s="34" t="s">
         <v>352</v>
-      </c>
-      <c r="E139" s="34" t="s">
-        <v>353</v>
       </c>
       <c r="F139" s="36"/>
       <c r="G139" s="36"/>
@@ -11330,10 +11341,10 @@
         <v>66</v>
       </c>
       <c r="D140" s="33" t="s">
+        <v>353</v>
+      </c>
+      <c r="E140" s="34" t="s">
         <v>354</v>
-      </c>
-      <c r="E140" s="34" t="s">
-        <v>355</v>
       </c>
       <c r="F140" s="36"/>
       <c r="G140" s="36"/>
@@ -11367,10 +11378,10 @@
         <v>66</v>
       </c>
       <c r="D141" s="33" t="s">
+        <v>355</v>
+      </c>
+      <c r="E141" s="34" t="s">
         <v>356</v>
-      </c>
-      <c r="E141" s="34" t="s">
-        <v>357</v>
       </c>
       <c r="F141" s="36"/>
       <c r="G141" s="36"/>
@@ -11404,10 +11415,10 @@
         <v>66</v>
       </c>
       <c r="D142" s="33" t="s">
+        <v>357</v>
+      </c>
+      <c r="E142" s="34" t="s">
         <v>358</v>
-      </c>
-      <c r="E142" s="34" t="s">
-        <v>359</v>
       </c>
       <c r="F142" s="36"/>
       <c r="G142" s="36"/>
@@ -11441,10 +11452,10 @@
         <v>66</v>
       </c>
       <c r="D143" s="33" t="s">
+        <v>359</v>
+      </c>
+      <c r="E143" s="34" t="s">
         <v>360</v>
-      </c>
-      <c r="E143" s="34" t="s">
-        <v>361</v>
       </c>
       <c r="F143" s="36"/>
       <c r="G143" s="36"/>
@@ -11478,10 +11489,10 @@
         <v>66</v>
       </c>
       <c r="D144" s="33" t="s">
+        <v>361</v>
+      </c>
+      <c r="E144" s="34" t="s">
         <v>362</v>
-      </c>
-      <c r="E144" s="34" t="s">
-        <v>363</v>
       </c>
       <c r="F144" s="36"/>
       <c r="G144" s="36"/>
@@ -11515,10 +11526,10 @@
         <v>66</v>
       </c>
       <c r="D145" s="33" t="s">
+        <v>363</v>
+      </c>
+      <c r="E145" s="34" t="s">
         <v>364</v>
-      </c>
-      <c r="E145" s="34" t="s">
-        <v>365</v>
       </c>
       <c r="F145" s="36"/>
       <c r="G145" s="36"/>
@@ -11552,23 +11563,23 @@
         <v>47</v>
       </c>
       <c r="D146" s="33" t="s">
+        <v>365</v>
+      </c>
+      <c r="E146" s="34" t="s">
         <v>366</v>
-      </c>
-      <c r="E146" s="34" t="s">
-        <v>367</v>
       </c>
       <c r="F146" s="36"/>
       <c r="G146" s="36"/>
       <c r="H146" s="36"/>
       <c r="I146" s="41"/>
       <c r="J146" s="42" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K146" s="42" t="s">
+        <v>367</v>
+      </c>
+      <c r="L146" s="42" t="s">
         <v>368</v>
-      </c>
-      <c r="L146" s="42" t="s">
-        <v>369</v>
       </c>
       <c r="M146" s="37"/>
       <c r="N146" s="37"/>
@@ -11595,23 +11606,23 @@
         <v>47</v>
       </c>
       <c r="D147" s="33" t="s">
+        <v>369</v>
+      </c>
+      <c r="E147" s="34" t="s">
         <v>370</v>
-      </c>
-      <c r="E147" s="34" t="s">
-        <v>371</v>
       </c>
       <c r="F147" s="36"/>
       <c r="G147" s="36"/>
       <c r="H147" s="36"/>
       <c r="I147" s="41"/>
       <c r="J147" s="42" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K147" s="42" t="s">
+        <v>367</v>
+      </c>
+      <c r="L147" s="42" t="s">
         <v>368</v>
-      </c>
-      <c r="L147" s="42" t="s">
-        <v>369</v>
       </c>
       <c r="M147" s="37"/>
       <c r="N147" s="37"/>
@@ -11635,13 +11646,13 @@
         <v>46</v>
       </c>
       <c r="C148" s="40" t="s">
+        <v>371</v>
+      </c>
+      <c r="D148" s="33" t="s">
         <v>372</v>
       </c>
-      <c r="D148" s="33" t="s">
+      <c r="E148" s="34" t="s">
         <v>373</v>
-      </c>
-      <c r="E148" s="34" t="s">
-        <v>374</v>
       </c>
       <c r="F148" s="36"/>
       <c r="G148" s="36"/>
@@ -11672,13 +11683,13 @@
         <v>46</v>
       </c>
       <c r="C149" s="40" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D149" s="33" t="s">
+        <v>374</v>
+      </c>
+      <c r="E149" s="34" t="s">
         <v>375</v>
-      </c>
-      <c r="E149" s="34" t="s">
-        <v>376</v>
       </c>
       <c r="F149" s="36"/>
       <c r="G149" s="36"/>
@@ -11709,13 +11720,13 @@
         <v>46</v>
       </c>
       <c r="C150" s="40" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D150" s="33" t="s">
+        <v>376</v>
+      </c>
+      <c r="E150" s="34" t="s">
         <v>377</v>
-      </c>
-      <c r="E150" s="34" t="s">
-        <v>378</v>
       </c>
       <c r="F150" s="36"/>
       <c r="G150" s="36"/>
@@ -11746,13 +11757,13 @@
         <v>46</v>
       </c>
       <c r="C151" s="40" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D151" s="33" t="s">
+        <v>378</v>
+      </c>
+      <c r="E151" s="34" t="s">
         <v>379</v>
-      </c>
-      <c r="E151" s="34" t="s">
-        <v>380</v>
       </c>
       <c r="F151" s="36"/>
       <c r="G151" s="36"/>
@@ -11783,13 +11794,13 @@
         <v>46</v>
       </c>
       <c r="C152" s="40" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D152" s="33" t="s">
+        <v>380</v>
+      </c>
+      <c r="E152" s="34" t="s">
         <v>381</v>
-      </c>
-      <c r="E152" s="34" t="s">
-        <v>382</v>
       </c>
       <c r="F152" s="36"/>
       <c r="G152" s="36"/>
@@ -11820,13 +11831,13 @@
         <v>46</v>
       </c>
       <c r="C153" s="40" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D153" s="33" t="s">
+        <v>382</v>
+      </c>
+      <c r="E153" s="34" t="s">
         <v>383</v>
-      </c>
-      <c r="E153" s="34" t="s">
-        <v>384</v>
       </c>
       <c r="F153" s="36"/>
       <c r="G153" s="36"/>
@@ -11859,13 +11870,13 @@
         <v>46</v>
       </c>
       <c r="C154" s="40" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D154" s="33" t="s">
+        <v>384</v>
+      </c>
+      <c r="E154" s="34" t="s">
         <v>385</v>
-      </c>
-      <c r="E154" s="34" t="s">
-        <v>386</v>
       </c>
       <c r="F154" s="36"/>
       <c r="G154" s="36"/>
@@ -11896,13 +11907,13 @@
         <v>46</v>
       </c>
       <c r="C155" s="40" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D155" s="33" t="s">
+        <v>386</v>
+      </c>
+      <c r="E155" s="34" t="s">
         <v>387</v>
-      </c>
-      <c r="E155" s="34" t="s">
-        <v>388</v>
       </c>
       <c r="F155" s="36"/>
       <c r="G155" s="36"/>
@@ -11933,13 +11944,13 @@
         <v>46</v>
       </c>
       <c r="C156" s="40" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D156" s="33" t="s">
+        <v>388</v>
+      </c>
+      <c r="E156" s="34" t="s">
         <v>389</v>
-      </c>
-      <c r="E156" s="34" t="s">
-        <v>390</v>
       </c>
       <c r="F156" s="36"/>
       <c r="G156" s="36"/>
@@ -11970,13 +11981,13 @@
         <v>46</v>
       </c>
       <c r="C157" s="40" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D157" s="33" t="s">
+        <v>390</v>
+      </c>
+      <c r="E157" s="34" t="s">
         <v>391</v>
-      </c>
-      <c r="E157" s="34" t="s">
-        <v>392</v>
       </c>
       <c r="F157" s="36"/>
       <c r="G157" s="36"/>
@@ -12007,13 +12018,13 @@
         <v>46</v>
       </c>
       <c r="C158" s="40" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D158" s="33" t="s">
+        <v>392</v>
+      </c>
+      <c r="E158" s="34" t="s">
         <v>393</v>
-      </c>
-      <c r="E158" s="34" t="s">
-        <v>394</v>
       </c>
       <c r="F158" s="36"/>
       <c r="G158" s="36"/>
@@ -12044,13 +12055,13 @@
         <v>46</v>
       </c>
       <c r="C159" s="40" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D159" s="33" t="s">
+        <v>394</v>
+      </c>
+      <c r="E159" s="34" t="s">
         <v>395</v>
-      </c>
-      <c r="E159" s="34" t="s">
-        <v>396</v>
       </c>
       <c r="F159" s="36"/>
       <c r="G159" s="36"/>
@@ -12081,13 +12092,13 @@
         <v>46</v>
       </c>
       <c r="C160" s="40" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D160" s="33" t="s">
+        <v>396</v>
+      </c>
+      <c r="E160" s="34" t="s">
         <v>397</v>
-      </c>
-      <c r="E160" s="34" t="s">
-        <v>398</v>
       </c>
       <c r="F160" s="36"/>
       <c r="G160" s="36"/>
@@ -12118,13 +12129,13 @@
         <v>46</v>
       </c>
       <c r="C161" s="40" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D161" s="33" t="s">
+        <v>398</v>
+      </c>
+      <c r="E161" s="34" t="s">
         <v>399</v>
-      </c>
-      <c r="E161" s="34" t="s">
-        <v>400</v>
       </c>
       <c r="F161" s="36"/>
       <c r="G161" s="36"/>
@@ -12155,13 +12166,13 @@
         <v>46</v>
       </c>
       <c r="C162" s="40" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D162" s="33" t="s">
+        <v>400</v>
+      </c>
+      <c r="E162" s="34" t="s">
         <v>401</v>
-      </c>
-      <c r="E162" s="34" t="s">
-        <v>402</v>
       </c>
       <c r="F162" s="36"/>
       <c r="G162" s="36"/>
@@ -12192,13 +12203,13 @@
         <v>46</v>
       </c>
       <c r="C163" s="40" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D163" s="33" t="s">
+        <v>402</v>
+      </c>
+      <c r="E163" s="34" t="s">
         <v>403</v>
-      </c>
-      <c r="E163" s="34" t="s">
-        <v>404</v>
       </c>
       <c r="F163" s="36"/>
       <c r="G163" s="36"/>
@@ -12232,10 +12243,10 @@
         <v>72</v>
       </c>
       <c r="D164" s="33" t="s">
+        <v>404</v>
+      </c>
+      <c r="E164" s="34" t="s">
         <v>405</v>
-      </c>
-      <c r="E164" s="34" t="s">
-        <v>406</v>
       </c>
       <c r="F164" s="36"/>
       <c r="G164" s="36"/>
@@ -12269,10 +12280,10 @@
         <v>72</v>
       </c>
       <c r="D165" s="33" t="s">
+        <v>406</v>
+      </c>
+      <c r="E165" s="34" t="s">
         <v>407</v>
-      </c>
-      <c r="E165" s="34" t="s">
-        <v>408</v>
       </c>
       <c r="F165" s="36"/>
       <c r="G165" s="36"/>
@@ -12306,10 +12317,10 @@
         <v>63</v>
       </c>
       <c r="D166" s="33" t="s">
+        <v>408</v>
+      </c>
+      <c r="E166" s="34" t="s">
         <v>409</v>
-      </c>
-      <c r="E166" s="34" t="s">
-        <v>410</v>
       </c>
       <c r="F166" s="36"/>
       <c r="G166" s="36"/>
@@ -12343,10 +12354,10 @@
         <v>63</v>
       </c>
       <c r="D167" s="33" t="s">
+        <v>410</v>
+      </c>
+      <c r="E167" s="34" t="s">
         <v>411</v>
-      </c>
-      <c r="E167" s="34" t="s">
-        <v>412</v>
       </c>
       <c r="F167" s="36"/>
       <c r="G167" s="36"/>
@@ -12380,22 +12391,22 @@
         <v>47</v>
       </c>
       <c r="D168" s="33" t="s">
+        <v>412</v>
+      </c>
+      <c r="E168" s="34" t="s">
         <v>413</v>
-      </c>
-      <c r="E168" s="34" t="s">
-        <v>414</v>
       </c>
       <c r="F168" s="36">
         <v>46093.0</v>
       </c>
       <c r="G168" s="36" t="s">
+        <v>414</v>
+      </c>
+      <c r="H168" s="36" t="s">
         <v>415</v>
       </c>
-      <c r="H168" s="36" t="s">
+      <c r="I168" s="41" t="s">
         <v>416</v>
-      </c>
-      <c r="I168" s="41" t="s">
-        <v>417</v>
       </c>
       <c r="J168" s="37" t="s">
         <v>53</v>
@@ -12427,10 +12438,10 @@
         <v>81</v>
       </c>
       <c r="D169" s="33" t="s">
+        <v>417</v>
+      </c>
+      <c r="E169" s="34" t="s">
         <v>418</v>
-      </c>
-      <c r="E169" s="34" t="s">
-        <v>419</v>
       </c>
       <c r="F169" s="36"/>
       <c r="G169" s="36"/>
@@ -12464,10 +12475,10 @@
         <v>81</v>
       </c>
       <c r="D170" s="33" t="s">
+        <v>419</v>
+      </c>
+      <c r="E170" s="34" t="s">
         <v>420</v>
-      </c>
-      <c r="E170" s="34" t="s">
-        <v>421</v>
       </c>
       <c r="F170" s="36"/>
       <c r="G170" s="36"/>
@@ -12501,10 +12512,10 @@
         <v>78</v>
       </c>
       <c r="D171" s="33" t="s">
+        <v>421</v>
+      </c>
+      <c r="E171" s="34" t="s">
         <v>422</v>
-      </c>
-      <c r="E171" s="34" t="s">
-        <v>423</v>
       </c>
       <c r="F171" s="36"/>
       <c r="G171" s="36"/>
@@ -12538,10 +12549,10 @@
         <v>78</v>
       </c>
       <c r="D172" s="33" t="s">
+        <v>423</v>
+      </c>
+      <c r="E172" s="34" t="s">
         <v>424</v>
-      </c>
-      <c r="E172" s="34" t="s">
-        <v>425</v>
       </c>
       <c r="F172" s="36"/>
       <c r="G172" s="36"/>
@@ -12575,10 +12586,10 @@
         <v>75</v>
       </c>
       <c r="D173" s="33" t="s">
+        <v>425</v>
+      </c>
+      <c r="E173" s="34" t="s">
         <v>426</v>
-      </c>
-      <c r="E173" s="34" t="s">
-        <v>427</v>
       </c>
       <c r="F173" s="36"/>
       <c r="G173" s="36"/>
@@ -12612,10 +12623,10 @@
         <v>75</v>
       </c>
       <c r="D174" s="33" t="s">
+        <v>427</v>
+      </c>
+      <c r="E174" s="34" t="s">
         <v>428</v>
-      </c>
-      <c r="E174" s="34" t="s">
-        <v>429</v>
       </c>
       <c r="F174" s="36"/>
       <c r="G174" s="36"/>
@@ -12646,13 +12657,13 @@
         <v>46</v>
       </c>
       <c r="C175" s="40" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D175" s="33" t="s">
+        <v>429</v>
+      </c>
+      <c r="E175" s="34" t="s">
         <v>430</v>
-      </c>
-      <c r="E175" s="34" t="s">
-        <v>431</v>
       </c>
       <c r="F175" s="36"/>
       <c r="G175" s="36"/>
@@ -12686,10 +12697,10 @@
         <v>72</v>
       </c>
       <c r="D176" s="33" t="s">
+        <v>431</v>
+      </c>
+      <c r="E176" s="34" t="s">
         <v>432</v>
-      </c>
-      <c r="E176" s="34" t="s">
-        <v>433</v>
       </c>
       <c r="F176" s="33"/>
       <c r="G176" s="33"/>
@@ -12723,10 +12734,10 @@
         <v>69</v>
       </c>
       <c r="D177" s="33" t="s">
+        <v>433</v>
+      </c>
+      <c r="E177" s="34" t="s">
         <v>434</v>
-      </c>
-      <c r="E177" s="34" t="s">
-        <v>435</v>
       </c>
       <c r="F177" s="33"/>
       <c r="G177" s="33"/>
@@ -12760,10 +12771,10 @@
         <v>81</v>
       </c>
       <c r="D178" s="33" t="s">
+        <v>435</v>
+      </c>
+      <c r="E178" s="34" t="s">
         <v>436</v>
-      </c>
-      <c r="E178" s="34" t="s">
-        <v>437</v>
       </c>
       <c r="F178" s="33"/>
       <c r="G178" s="33"/>
@@ -12797,10 +12808,10 @@
         <v>75</v>
       </c>
       <c r="D179" s="33" t="s">
+        <v>437</v>
+      </c>
+      <c r="E179" s="34" t="s">
         <v>438</v>
-      </c>
-      <c r="E179" s="34" t="s">
-        <v>439</v>
       </c>
       <c r="F179" s="33"/>
       <c r="G179" s="33"/>
@@ -12834,10 +12845,10 @@
         <v>78</v>
       </c>
       <c r="D180" s="33" t="s">
+        <v>439</v>
+      </c>
+      <c r="E180" s="34" t="s">
         <v>440</v>
-      </c>
-      <c r="E180" s="34" t="s">
-        <v>441</v>
       </c>
       <c r="F180" s="33"/>
       <c r="G180" s="33"/>
@@ -12860,7 +12871,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="181" ht="14.25" customHeight="1">
+    <row r="181">
       <c r="A181" s="33">
         <v>466.0</v>
       </c>
@@ -12871,22 +12882,22 @@
         <v>47</v>
       </c>
       <c r="D181" s="33" t="s">
+        <v>441</v>
+      </c>
+      <c r="E181" s="34" t="s">
         <v>442</v>
-      </c>
-      <c r="E181" s="34" t="s">
-        <v>443</v>
       </c>
       <c r="F181" s="36">
         <v>46094.0</v>
       </c>
       <c r="G181" s="33" t="s">
+        <v>443</v>
+      </c>
+      <c r="H181" s="33" t="s">
         <v>444</v>
       </c>
-      <c r="H181" s="33" t="s">
+      <c r="I181" s="33" t="s">
         <v>445</v>
-      </c>
-      <c r="I181" s="33" t="s">
-        <v>446</v>
       </c>
       <c r="J181" s="37" t="s">
         <v>53</v>
@@ -12899,19 +12910,21 @@
       <c r="N181" s="37" t="s">
         <v>53</v>
       </c>
-      <c r="O181" s="33" t="s">
-        <v>447</v>
+      <c r="O181" s="37" t="s">
+        <v>446</v>
       </c>
       <c r="P181" s="37" t="s">
         <v>53</v>
       </c>
       <c r="Q181" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="R181" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="S181" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="R181" s="37" t="s">
-        <v>61</v>
-      </c>
-      <c r="S181" s="33"/>
       <c r="T181" s="37"/>
       <c r="U181" s="33"/>
       <c r="V181" s="33"/>
@@ -12930,10 +12943,10 @@
         <v>63</v>
       </c>
       <c r="D182" s="33" t="s">
+        <v>447</v>
+      </c>
+      <c r="E182" s="34" t="s">
         <v>448</v>
-      </c>
-      <c r="E182" s="34" t="s">
-        <v>449</v>
       </c>
       <c r="F182" s="33"/>
       <c r="G182" s="33"/>
@@ -12967,10 +12980,10 @@
         <v>72</v>
       </c>
       <c r="D183" s="33" t="s">
+        <v>449</v>
+      </c>
+      <c r="E183" s="34" t="s">
         <v>450</v>
-      </c>
-      <c r="E183" s="34" t="s">
-        <v>451</v>
       </c>
       <c r="F183" s="33"/>
       <c r="G183" s="33"/>
@@ -13004,10 +13017,10 @@
         <v>66</v>
       </c>
       <c r="D184" s="33" t="s">
+        <v>451</v>
+      </c>
+      <c r="E184" s="34" t="s">
         <v>452</v>
-      </c>
-      <c r="E184" s="34" t="s">
-        <v>453</v>
       </c>
       <c r="F184" s="33"/>
       <c r="G184" s="33"/>
@@ -13038,13 +13051,13 @@
         <v>46</v>
       </c>
       <c r="C185" s="40" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D185" s="33" t="s">
+        <v>453</v>
+      </c>
+      <c r="E185" s="34" t="s">
         <v>454</v>
-      </c>
-      <c r="E185" s="34" t="s">
-        <v>455</v>
       </c>
       <c r="F185" s="33"/>
       <c r="G185" s="33"/>
@@ -13078,10 +13091,10 @@
         <v>69</v>
       </c>
       <c r="D186" s="33" t="s">
+        <v>455</v>
+      </c>
+      <c r="E186" s="34" t="s">
         <v>456</v>
-      </c>
-      <c r="E186" s="34" t="s">
-        <v>457</v>
       </c>
       <c r="F186" s="36"/>
       <c r="G186" s="36"/>
@@ -13115,10 +13128,10 @@
         <v>69</v>
       </c>
       <c r="D187" s="33" t="s">
+        <v>457</v>
+      </c>
+      <c r="E187" s="34" t="s">
         <v>458</v>
-      </c>
-      <c r="E187" s="34" t="s">
-        <v>459</v>
       </c>
       <c r="F187" s="36"/>
       <c r="G187" s="36"/>
@@ -13141,7 +13154,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="188" ht="14.25" customHeight="1">
+    <row r="188">
       <c r="A188" s="33">
         <v>473.0</v>
       </c>
@@ -13152,22 +13165,22 @@
         <v>47</v>
       </c>
       <c r="D188" s="40" t="s">
+        <v>459</v>
+      </c>
+      <c r="E188" s="34" t="s">
         <v>460</v>
-      </c>
-      <c r="E188" s="34" t="s">
-        <v>461</v>
       </c>
       <c r="F188" s="36">
         <v>46094.0</v>
       </c>
       <c r="G188" s="36" t="s">
+        <v>461</v>
+      </c>
+      <c r="H188" s="36" t="s">
         <v>462</v>
       </c>
-      <c r="H188" s="36" t="s">
+      <c r="I188" s="41" t="s">
         <v>463</v>
-      </c>
-      <c r="I188" s="41" t="s">
-        <v>464</v>
       </c>
       <c r="J188" s="37" t="s">
         <v>53</v>
@@ -13179,18 +13192,20 @@
       </c>
       <c r="N188" s="37"/>
       <c r="O188" s="37" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="P188" s="37" t="s">
         <v>53</v>
       </c>
       <c r="Q188" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="R188" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="S188" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="R188" s="37" t="s">
-        <v>61</v>
-      </c>
-      <c r="S188" s="37"/>
       <c r="T188" s="37"/>
       <c r="U188" s="38"/>
       <c r="V188" s="39"/>
@@ -13209,10 +13224,10 @@
         <v>69</v>
       </c>
       <c r="D189" s="33" t="s">
+        <v>465</v>
+      </c>
+      <c r="E189" s="34" t="s">
         <v>466</v>
-      </c>
-      <c r="E189" s="34" t="s">
-        <v>467</v>
       </c>
       <c r="F189" s="36"/>
       <c r="G189" s="36"/>
@@ -13246,10 +13261,10 @@
         <v>72</v>
       </c>
       <c r="D190" s="33" t="s">
+        <v>467</v>
+      </c>
+      <c r="E190" s="34" t="s">
         <v>468</v>
-      </c>
-      <c r="E190" s="34" t="s">
-        <v>469</v>
       </c>
       <c r="F190" s="36"/>
       <c r="G190" s="36"/>
@@ -13283,10 +13298,10 @@
         <v>66</v>
       </c>
       <c r="D191" s="33" t="s">
+        <v>469</v>
+      </c>
+      <c r="E191" s="34" t="s">
         <v>470</v>
-      </c>
-      <c r="E191" s="34" t="s">
-        <v>471</v>
       </c>
       <c r="F191" s="36"/>
       <c r="G191" s="36"/>
@@ -13320,10 +13335,10 @@
         <v>66</v>
       </c>
       <c r="D192" s="33" t="s">
+        <v>471</v>
+      </c>
+      <c r="E192" s="34" t="s">
         <v>472</v>
-      </c>
-      <c r="E192" s="34" t="s">
-        <v>473</v>
       </c>
       <c r="F192" s="36"/>
       <c r="G192" s="36"/>
@@ -13357,10 +13372,10 @@
         <v>66</v>
       </c>
       <c r="D193" s="33" t="s">
+        <v>473</v>
+      </c>
+      <c r="E193" s="34" t="s">
         <v>474</v>
-      </c>
-      <c r="E193" s="34" t="s">
-        <v>475</v>
       </c>
       <c r="F193" s="36"/>
       <c r="G193" s="36"/>
@@ -13391,13 +13406,13 @@
         <v>46</v>
       </c>
       <c r="C194" s="40" t="s">
+        <v>475</v>
+      </c>
+      <c r="D194" s="33" t="s">
         <v>476</v>
       </c>
-      <c r="D194" s="33" t="s">
+      <c r="E194" s="34" t="s">
         <v>477</v>
-      </c>
-      <c r="E194" s="34" t="s">
-        <v>478</v>
       </c>
       <c r="F194" s="36"/>
       <c r="G194" s="36"/>
@@ -13428,13 +13443,13 @@
         <v>46</v>
       </c>
       <c r="C195" s="40" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="D195" s="33" t="s">
+        <v>478</v>
+      </c>
+      <c r="E195" s="34" t="s">
         <v>479</v>
-      </c>
-      <c r="E195" s="34" t="s">
-        <v>480</v>
       </c>
       <c r="F195" s="36"/>
       <c r="G195" s="36"/>
@@ -13465,13 +13480,13 @@
         <v>46</v>
       </c>
       <c r="C196" s="40" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="D196" s="33" t="s">
+        <v>480</v>
+      </c>
+      <c r="E196" s="34" t="s">
         <v>481</v>
-      </c>
-      <c r="E196" s="34" t="s">
-        <v>482</v>
       </c>
       <c r="F196" s="36"/>
       <c r="G196" s="36"/>
@@ -13502,13 +13517,13 @@
         <v>46</v>
       </c>
       <c r="C197" s="40" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="D197" s="33" t="s">
+        <v>482</v>
+      </c>
+      <c r="E197" s="34" t="s">
         <v>483</v>
-      </c>
-      <c r="E197" s="34" t="s">
-        <v>484</v>
       </c>
       <c r="F197" s="36"/>
       <c r="G197" s="36"/>
@@ -13539,13 +13554,13 @@
         <v>46</v>
       </c>
       <c r="C198" s="40" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="D198" s="33" t="s">
+        <v>484</v>
+      </c>
+      <c r="E198" s="34" t="s">
         <v>485</v>
-      </c>
-      <c r="E198" s="34" t="s">
-        <v>486</v>
       </c>
       <c r="F198" s="36"/>
       <c r="G198" s="36"/>
@@ -13576,13 +13591,13 @@
         <v>46</v>
       </c>
       <c r="C199" s="40" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="D199" s="33" t="s">
+        <v>486</v>
+      </c>
+      <c r="E199" s="34" t="s">
         <v>487</v>
-      </c>
-      <c r="E199" s="34" t="s">
-        <v>488</v>
       </c>
       <c r="F199" s="36"/>
       <c r="G199" s="36"/>
@@ -13613,13 +13628,13 @@
         <v>46</v>
       </c>
       <c r="C200" s="40" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="D200" s="33" t="s">
+        <v>488</v>
+      </c>
+      <c r="E200" s="34" t="s">
         <v>489</v>
-      </c>
-      <c r="E200" s="34" t="s">
-        <v>490</v>
       </c>
       <c r="F200" s="36"/>
       <c r="G200" s="36"/>
@@ -13650,13 +13665,13 @@
         <v>46</v>
       </c>
       <c r="C201" s="40" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="D201" s="33" t="s">
+        <v>490</v>
+      </c>
+      <c r="E201" s="34" t="s">
         <v>491</v>
-      </c>
-      <c r="E201" s="34" t="s">
-        <v>492</v>
       </c>
       <c r="F201" s="36"/>
       <c r="G201" s="36"/>
@@ -13687,13 +13702,13 @@
         <v>46</v>
       </c>
       <c r="C202" s="40" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="D202" s="33" t="s">
+        <v>492</v>
+      </c>
+      <c r="E202" s="34" t="s">
         <v>493</v>
-      </c>
-      <c r="E202" s="34" t="s">
-        <v>494</v>
       </c>
       <c r="F202" s="36"/>
       <c r="G202" s="36"/>
@@ -13724,13 +13739,13 @@
         <v>46</v>
       </c>
       <c r="C203" s="40" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="D203" s="33" t="s">
+        <v>494</v>
+      </c>
+      <c r="E203" s="34" t="s">
         <v>495</v>
-      </c>
-      <c r="E203" s="34" t="s">
-        <v>496</v>
       </c>
       <c r="F203" s="36"/>
       <c r="G203" s="36"/>
@@ -13761,13 +13776,13 @@
         <v>46</v>
       </c>
       <c r="C204" s="40" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="D204" s="33" t="s">
+        <v>496</v>
+      </c>
+      <c r="E204" s="34" t="s">
         <v>497</v>
-      </c>
-      <c r="E204" s="34" t="s">
-        <v>498</v>
       </c>
       <c r="F204" s="36"/>
       <c r="G204" s="36"/>
@@ -13798,10 +13813,10 @@
         <v>46</v>
       </c>
       <c r="C205" s="40" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="D205" s="33" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="E205" s="34" t="s">
         <v>104</v>
@@ -13837,13 +13852,13 @@
         <v>46</v>
       </c>
       <c r="C206" s="40" t="s">
+        <v>499</v>
+      </c>
+      <c r="D206" s="33" t="s">
         <v>500</v>
       </c>
-      <c r="D206" s="33" t="s">
+      <c r="E206" s="34" t="s">
         <v>501</v>
-      </c>
-      <c r="E206" s="34" t="s">
-        <v>502</v>
       </c>
       <c r="F206" s="36"/>
       <c r="G206" s="36"/>
@@ -13874,13 +13889,13 @@
         <v>46</v>
       </c>
       <c r="C207" s="40" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="D207" s="33" t="s">
+        <v>502</v>
+      </c>
+      <c r="E207" s="34" t="s">
         <v>503</v>
-      </c>
-      <c r="E207" s="34" t="s">
-        <v>504</v>
       </c>
       <c r="F207" s="36"/>
       <c r="G207" s="36"/>
@@ -13911,13 +13926,13 @@
         <v>46</v>
       </c>
       <c r="C208" s="40" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="D208" s="33" t="s">
+        <v>504</v>
+      </c>
+      <c r="E208" s="34" t="s">
         <v>505</v>
-      </c>
-      <c r="E208" s="34" t="s">
-        <v>506</v>
       </c>
       <c r="F208" s="36"/>
       <c r="G208" s="36"/>
@@ -13948,13 +13963,13 @@
         <v>46</v>
       </c>
       <c r="C209" s="40" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="D209" s="33" t="s">
+        <v>506</v>
+      </c>
+      <c r="E209" s="34" t="s">
         <v>507</v>
-      </c>
-      <c r="E209" s="34" t="s">
-        <v>508</v>
       </c>
       <c r="F209" s="36"/>
       <c r="G209" s="36"/>
@@ -13985,13 +14000,13 @@
         <v>46</v>
       </c>
       <c r="C210" s="40" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="D210" s="33" t="s">
+        <v>508</v>
+      </c>
+      <c r="E210" s="34" t="s">
         <v>509</v>
-      </c>
-      <c r="E210" s="34" t="s">
-        <v>510</v>
       </c>
       <c r="F210" s="36"/>
       <c r="G210" s="36"/>
@@ -14022,13 +14037,13 @@
         <v>46</v>
       </c>
       <c r="C211" s="40" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="D211" s="33" t="s">
+        <v>510</v>
+      </c>
+      <c r="E211" s="34" t="s">
         <v>511</v>
-      </c>
-      <c r="E211" s="34" t="s">
-        <v>512</v>
       </c>
       <c r="F211" s="36"/>
       <c r="G211" s="36"/>
@@ -14059,13 +14074,13 @@
         <v>46</v>
       </c>
       <c r="C212" s="40" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="D212" s="33" t="s">
+        <v>512</v>
+      </c>
+      <c r="E212" s="34" t="s">
         <v>513</v>
-      </c>
-      <c r="E212" s="34" t="s">
-        <v>514</v>
       </c>
       <c r="F212" s="36"/>
       <c r="G212" s="36"/>
@@ -14096,13 +14111,13 @@
         <v>46</v>
       </c>
       <c r="C213" s="40" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="D213" s="33" t="s">
+        <v>514</v>
+      </c>
+      <c r="E213" s="34" t="s">
         <v>515</v>
-      </c>
-      <c r="E213" s="34" t="s">
-        <v>516</v>
       </c>
       <c r="F213" s="36"/>
       <c r="G213" s="36"/>
@@ -14133,13 +14148,13 @@
         <v>46</v>
       </c>
       <c r="C214" s="40" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="D214" s="33" t="s">
+        <v>516</v>
+      </c>
+      <c r="E214" s="34" t="s">
         <v>517</v>
-      </c>
-      <c r="E214" s="34" t="s">
-        <v>518</v>
       </c>
       <c r="F214" s="36"/>
       <c r="G214" s="36"/>
@@ -14170,13 +14185,13 @@
         <v>46</v>
       </c>
       <c r="C215" s="40" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="D215" s="33" t="s">
+        <v>518</v>
+      </c>
+      <c r="E215" s="34" t="s">
         <v>519</v>
-      </c>
-      <c r="E215" s="34" t="s">
-        <v>520</v>
       </c>
       <c r="F215" s="36"/>
       <c r="G215" s="36"/>
@@ -14207,13 +14222,13 @@
         <v>46</v>
       </c>
       <c r="C216" s="40" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="D216" s="33" t="s">
+        <v>520</v>
+      </c>
+      <c r="E216" s="34" t="s">
         <v>521</v>
-      </c>
-      <c r="E216" s="34" t="s">
-        <v>522</v>
       </c>
       <c r="F216" s="36"/>
       <c r="G216" s="36"/>
@@ -14244,13 +14259,13 @@
         <v>46</v>
       </c>
       <c r="C217" s="40" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="D217" s="33" t="s">
+        <v>522</v>
+      </c>
+      <c r="E217" s="34" t="s">
         <v>523</v>
-      </c>
-      <c r="E217" s="34" t="s">
-        <v>524</v>
       </c>
       <c r="F217" s="36"/>
       <c r="G217" s="36"/>
@@ -14281,13 +14296,13 @@
         <v>46</v>
       </c>
       <c r="C218" s="40" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="D218" s="33" t="s">
+        <v>524</v>
+      </c>
+      <c r="E218" s="34" t="s">
         <v>525</v>
-      </c>
-      <c r="E218" s="34" t="s">
-        <v>526</v>
       </c>
       <c r="F218" s="36"/>
       <c r="G218" s="36"/>
@@ -14318,13 +14333,13 @@
         <v>46</v>
       </c>
       <c r="C219" s="40" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="D219" s="33" t="s">
+        <v>526</v>
+      </c>
+      <c r="E219" s="34" t="s">
         <v>527</v>
-      </c>
-      <c r="E219" s="34" t="s">
-        <v>528</v>
       </c>
       <c r="F219" s="36"/>
       <c r="G219" s="36"/>
@@ -14355,10 +14370,10 @@
         <v>46</v>
       </c>
       <c r="C220" s="40" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="D220" s="33" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="E220" s="34" t="s">
         <v>104</v>
@@ -14394,13 +14409,13 @@
         <v>46</v>
       </c>
       <c r="C221" s="40" t="s">
+        <v>529</v>
+      </c>
+      <c r="D221" s="33" t="s">
         <v>530</v>
       </c>
-      <c r="D221" s="33" t="s">
+      <c r="E221" s="34" t="s">
         <v>531</v>
-      </c>
-      <c r="E221" s="34" t="s">
-        <v>532</v>
       </c>
       <c r="F221" s="36"/>
       <c r="G221" s="36"/>
@@ -14431,13 +14446,13 @@
         <v>46</v>
       </c>
       <c r="C222" s="40" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="D222" s="33" t="s">
+        <v>532</v>
+      </c>
+      <c r="E222" s="34" t="s">
         <v>533</v>
-      </c>
-      <c r="E222" s="34" t="s">
-        <v>534</v>
       </c>
       <c r="F222" s="36"/>
       <c r="G222" s="36"/>
@@ -14468,13 +14483,13 @@
         <v>46</v>
       </c>
       <c r="C223" s="40" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="D223" s="33" t="s">
+        <v>534</v>
+      </c>
+      <c r="E223" s="34" t="s">
         <v>535</v>
-      </c>
-      <c r="E223" s="34" t="s">
-        <v>536</v>
       </c>
       <c r="F223" s="36"/>
       <c r="G223" s="36"/>
@@ -14505,13 +14520,13 @@
         <v>46</v>
       </c>
       <c r="C224" s="40" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="D224" s="33" t="s">
+        <v>536</v>
+      </c>
+      <c r="E224" s="34" t="s">
         <v>537</v>
-      </c>
-      <c r="E224" s="34" t="s">
-        <v>538</v>
       </c>
       <c r="F224" s="36"/>
       <c r="G224" s="36"/>
@@ -14542,13 +14557,13 @@
         <v>46</v>
       </c>
       <c r="C225" s="40" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="D225" s="33" t="s">
+        <v>538</v>
+      </c>
+      <c r="E225" s="34" t="s">
         <v>539</v>
-      </c>
-      <c r="E225" s="34" t="s">
-        <v>540</v>
       </c>
       <c r="F225" s="36"/>
       <c r="G225" s="36"/>
@@ -14579,13 +14594,13 @@
         <v>46</v>
       </c>
       <c r="C226" s="40" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="D226" s="33" t="s">
+        <v>540</v>
+      </c>
+      <c r="E226" s="34" t="s">
         <v>541</v>
-      </c>
-      <c r="E226" s="34" t="s">
-        <v>542</v>
       </c>
       <c r="F226" s="36"/>
       <c r="G226" s="36"/>
@@ -14616,13 +14631,13 @@
         <v>46</v>
       </c>
       <c r="C227" s="40" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="D227" s="33" t="s">
+        <v>542</v>
+      </c>
+      <c r="E227" s="34" t="s">
         <v>543</v>
-      </c>
-      <c r="E227" s="34" t="s">
-        <v>544</v>
       </c>
       <c r="F227" s="36"/>
       <c r="G227" s="36"/>
@@ -14653,13 +14668,13 @@
         <v>46</v>
       </c>
       <c r="C228" s="40" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="D228" s="33" t="s">
+        <v>544</v>
+      </c>
+      <c r="E228" s="34" t="s">
         <v>545</v>
-      </c>
-      <c r="E228" s="34" t="s">
-        <v>546</v>
       </c>
       <c r="F228" s="36"/>
       <c r="G228" s="36"/>
@@ -14690,13 +14705,13 @@
         <v>46</v>
       </c>
       <c r="C229" s="40" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="D229" s="33" t="s">
+        <v>546</v>
+      </c>
+      <c r="E229" s="34" t="s">
         <v>547</v>
-      </c>
-      <c r="E229" s="34" t="s">
-        <v>548</v>
       </c>
       <c r="F229" s="36"/>
       <c r="G229" s="36"/>
@@ -14727,13 +14742,13 @@
         <v>46</v>
       </c>
       <c r="C230" s="40" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="D230" s="33" t="s">
+        <v>548</v>
+      </c>
+      <c r="E230" s="34" t="s">
         <v>549</v>
-      </c>
-      <c r="E230" s="34" t="s">
-        <v>550</v>
       </c>
       <c r="F230" s="36"/>
       <c r="G230" s="36"/>
@@ -14764,13 +14779,13 @@
         <v>46</v>
       </c>
       <c r="C231" s="40" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="D231" s="33" t="s">
+        <v>550</v>
+      </c>
+      <c r="E231" s="34" t="s">
         <v>551</v>
-      </c>
-      <c r="E231" s="34" t="s">
-        <v>552</v>
       </c>
       <c r="F231" s="36"/>
       <c r="G231" s="36"/>
@@ -14801,13 +14816,13 @@
         <v>46</v>
       </c>
       <c r="C232" s="40" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="D232" s="33" t="s">
+        <v>552</v>
+      </c>
+      <c r="E232" s="34" t="s">
         <v>553</v>
-      </c>
-      <c r="E232" s="34" t="s">
-        <v>554</v>
       </c>
       <c r="F232" s="36"/>
       <c r="G232" s="36"/>
@@ -14838,13 +14853,13 @@
         <v>46</v>
       </c>
       <c r="C233" s="40" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="D233" s="33" t="s">
+        <v>554</v>
+      </c>
+      <c r="E233" s="34" t="s">
         <v>555</v>
-      </c>
-      <c r="E233" s="34" t="s">
-        <v>556</v>
       </c>
       <c r="F233" s="36"/>
       <c r="G233" s="36"/>
@@ -14875,13 +14890,13 @@
         <v>46</v>
       </c>
       <c r="C234" s="40" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="D234" s="33" t="s">
+        <v>556</v>
+      </c>
+      <c r="E234" s="34" t="s">
         <v>557</v>
-      </c>
-      <c r="E234" s="34" t="s">
-        <v>558</v>
       </c>
       <c r="F234" s="36"/>
       <c r="G234" s="36"/>
@@ -14912,10 +14927,10 @@
         <v>46</v>
       </c>
       <c r="C235" s="40" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="D235" s="33" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="E235" s="34" t="s">
         <v>104</v>
@@ -14951,13 +14966,13 @@
         <v>46</v>
       </c>
       <c r="C236" s="40" t="s">
+        <v>559</v>
+      </c>
+      <c r="D236" s="33" t="s">
         <v>560</v>
       </c>
-      <c r="D236" s="33" t="s">
+      <c r="E236" s="34" t="s">
         <v>561</v>
-      </c>
-      <c r="E236" s="34" t="s">
-        <v>562</v>
       </c>
       <c r="F236" s="36"/>
       <c r="G236" s="36"/>
@@ -14988,13 +15003,13 @@
         <v>46</v>
       </c>
       <c r="C237" s="40" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="D237" s="33" t="s">
+        <v>562</v>
+      </c>
+      <c r="E237" s="34" t="s">
         <v>563</v>
-      </c>
-      <c r="E237" s="34" t="s">
-        <v>564</v>
       </c>
       <c r="F237" s="36"/>
       <c r="G237" s="36"/>
@@ -15025,13 +15040,13 @@
         <v>46</v>
       </c>
       <c r="C238" s="40" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="D238" s="33" t="s">
+        <v>564</v>
+      </c>
+      <c r="E238" s="34" t="s">
         <v>565</v>
-      </c>
-      <c r="E238" s="34" t="s">
-        <v>566</v>
       </c>
       <c r="F238" s="36"/>
       <c r="G238" s="36"/>
@@ -15062,13 +15077,13 @@
         <v>46</v>
       </c>
       <c r="C239" s="40" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="D239" s="33" t="s">
+        <v>566</v>
+      </c>
+      <c r="E239" s="34" t="s">
         <v>567</v>
-      </c>
-      <c r="E239" s="34" t="s">
-        <v>568</v>
       </c>
       <c r="F239" s="36"/>
       <c r="G239" s="36"/>
@@ -15099,13 +15114,13 @@
         <v>46</v>
       </c>
       <c r="C240" s="40" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="D240" s="33" t="s">
+        <v>568</v>
+      </c>
+      <c r="E240" s="34" t="s">
         <v>569</v>
-      </c>
-      <c r="E240" s="34" t="s">
-        <v>570</v>
       </c>
       <c r="F240" s="36"/>
       <c r="G240" s="36"/>
@@ -15136,13 +15151,13 @@
         <v>46</v>
       </c>
       <c r="C241" s="40" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="D241" s="33" t="s">
+        <v>570</v>
+      </c>
+      <c r="E241" s="34" t="s">
         <v>571</v>
-      </c>
-      <c r="E241" s="34" t="s">
-        <v>572</v>
       </c>
       <c r="F241" s="36"/>
       <c r="G241" s="36"/>
@@ -15173,13 +15188,13 @@
         <v>46</v>
       </c>
       <c r="C242" s="40" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="D242" s="33" t="s">
+        <v>572</v>
+      </c>
+      <c r="E242" s="34" t="s">
         <v>573</v>
-      </c>
-      <c r="E242" s="34" t="s">
-        <v>574</v>
       </c>
       <c r="F242" s="36"/>
       <c r="G242" s="36"/>
@@ -15210,13 +15225,13 @@
         <v>46</v>
       </c>
       <c r="C243" s="40" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="D243" s="33" t="s">
+        <v>574</v>
+      </c>
+      <c r="E243" s="34" t="s">
         <v>575</v>
-      </c>
-      <c r="E243" s="34" t="s">
-        <v>576</v>
       </c>
       <c r="F243" s="36"/>
       <c r="G243" s="36"/>
@@ -15247,13 +15262,13 @@
         <v>46</v>
       </c>
       <c r="C244" s="40" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="D244" s="33" t="s">
+        <v>576</v>
+      </c>
+      <c r="E244" s="34" t="s">
         <v>577</v>
-      </c>
-      <c r="E244" s="34" t="s">
-        <v>578</v>
       </c>
       <c r="F244" s="36"/>
       <c r="G244" s="36"/>
@@ -15284,10 +15299,10 @@
         <v>46</v>
       </c>
       <c r="C245" s="40" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="D245" s="33" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="E245" s="34" t="s">
         <v>104</v>
@@ -18333,42 +18348,42 @@
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
       <c r="A1" s="44" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="44" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="44" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="44" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="44" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="44" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="44" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
       <c r="A8" s="44" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1"/>
@@ -19389,22 +19404,22 @@
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
       <c r="A1" s="45" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="B1" s="46" t="s">
         <v>24</v>
       </c>
       <c r="C1" s="46" t="s">
+        <v>587</v>
+      </c>
+      <c r="D1" s="46" t="s">
         <v>588</v>
       </c>
-      <c r="D1" s="46" t="s">
+      <c r="F1" s="47" t="s">
         <v>589</v>
       </c>
-      <c r="F1" s="47" t="s">
+      <c r="G1" s="48" t="s">
         <v>590</v>
-      </c>
-      <c r="G1" s="48" t="s">
-        <v>591</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
@@ -19412,13 +19427,13 @@
         <v>47</v>
       </c>
       <c r="B2" s="49" t="s">
+        <v>591</v>
+      </c>
+      <c r="C2" s="50" t="s">
         <v>592</v>
       </c>
-      <c r="C2" s="50" t="s">
+      <c r="D2" s="50" t="s">
         <v>593</v>
-      </c>
-      <c r="D2" s="50" t="s">
-        <v>594</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
@@ -19426,13 +19441,13 @@
         <v>63</v>
       </c>
       <c r="B3" s="49" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="C3" s="50" t="s">
+        <v>594</v>
+      </c>
+      <c r="D3" s="50" t="s">
         <v>595</v>
-      </c>
-      <c r="D3" s="50" t="s">
-        <v>596</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
@@ -19440,13 +19455,13 @@
         <v>69</v>
       </c>
       <c r="B4" s="49" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="C4" s="50" t="s">
+        <v>596</v>
+      </c>
+      <c r="D4" s="51" t="s">
         <v>597</v>
-      </c>
-      <c r="D4" s="51" t="s">
-        <v>598</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
@@ -19454,13 +19469,13 @@
         <v>75</v>
       </c>
       <c r="B5" s="49" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="C5" s="50" t="s">
+        <v>598</v>
+      </c>
+      <c r="D5" s="50" t="s">
         <v>599</v>
-      </c>
-      <c r="D5" s="50" t="s">
-        <v>600</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
@@ -19468,13 +19483,13 @@
         <v>78</v>
       </c>
       <c r="B6" s="49" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="C6" s="50" t="s">
+        <v>600</v>
+      </c>
+      <c r="D6" s="51" t="s">
         <v>601</v>
-      </c>
-      <c r="D6" s="51" t="s">
-        <v>602</v>
       </c>
     </row>
     <row r="7">
@@ -19482,13 +19497,13 @@
         <v>81</v>
       </c>
       <c r="B7" s="49" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="C7" s="50" t="s">
+        <v>602</v>
+      </c>
+      <c r="D7" s="51" t="s">
         <v>603</v>
-      </c>
-      <c r="D7" s="51" t="s">
-        <v>604</v>
       </c>
     </row>
     <row r="8">
@@ -19496,13 +19511,13 @@
         <v>72</v>
       </c>
       <c r="B8" s="49" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="C8" s="50" t="s">
+        <v>604</v>
+      </c>
+      <c r="D8" s="51" t="s">
         <v>605</v>
-      </c>
-      <c r="D8" s="51" t="s">
-        <v>606</v>
       </c>
     </row>
     <row r="9">
@@ -19510,97 +19525,97 @@
         <v>66</v>
       </c>
       <c r="B9" s="49" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="C9" s="50" t="s">
+        <v>606</v>
+      </c>
+      <c r="D9" s="51" t="s">
         <v>607</v>
-      </c>
-      <c r="D9" s="51" t="s">
-        <v>608</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="49" t="s">
+        <v>608</v>
+      </c>
+      <c r="B10" s="49" t="s">
+        <v>591</v>
+      </c>
+      <c r="C10" s="51" t="s">
         <v>609</v>
       </c>
-      <c r="B10" s="49" t="s">
-        <v>592</v>
-      </c>
-      <c r="C10" s="51" t="s">
+      <c r="D10" s="50" t="s">
         <v>610</v>
-      </c>
-      <c r="D10" s="50" t="s">
-        <v>611</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
       <c r="A11" s="49" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B11" s="49" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="C11" s="50" t="s">
+        <v>611</v>
+      </c>
+      <c r="D11" s="51" t="s">
         <v>612</v>
-      </c>
-      <c r="D11" s="51" t="s">
-        <v>613</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="49" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B12" s="49" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="C12" s="50" t="s">
+        <v>613</v>
+      </c>
+      <c r="D12" s="51" t="s">
         <v>614</v>
-      </c>
-      <c r="D12" s="51" t="s">
-        <v>615</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="49" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="B13" s="49" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="C13" s="50" t="s">
+        <v>615</v>
+      </c>
+      <c r="D13" s="51" t="s">
         <v>616</v>
-      </c>
-      <c r="D13" s="51" t="s">
-        <v>617</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
       <c r="A14" s="49" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B14" s="49" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="C14" s="50" t="s">
+        <v>617</v>
+      </c>
+      <c r="D14" s="51" t="s">
         <v>618</v>
-      </c>
-      <c r="D14" s="51" t="s">
-        <v>619</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="49" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="B15" s="49" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="C15" s="50">
         <v>521.0</v>
       </c>
       <c r="D15" s="51" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1">
@@ -22589,7 +22604,7 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="52" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="B2" s="52" t="s">
         <v>53</v>
@@ -22597,10 +22612,10 @@
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="52" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B3" s="52" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">

</xml_diff>

<commit_message>
Compilazione colonna S caso 55 e N caso 473
Compilazione colonna S caso 55 e colonna N caso 473.
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#ENTERXX/it.entersrl/it.entersrl.extralab/4.15.4.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#ENTERXX/it.entersrl/it.entersrl.extralab/4.15.4.0/report-checklist.xlsx
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1462" uniqueCount="622">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1464" uniqueCount="622">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -7371,7 +7371,9 @@
       <c r="R36" s="37" t="s">
         <v>60</v>
       </c>
-      <c r="S36" s="37"/>
+      <c r="S36" s="42" t="s">
+        <v>61</v>
+      </c>
       <c r="T36" s="37"/>
       <c r="U36" s="38"/>
       <c r="V36" s="39"/>
@@ -13190,7 +13192,9 @@
       <c r="M188" s="37" t="s">
         <v>53</v>
       </c>
-      <c r="N188" s="37"/>
+      <c r="N188" s="42" t="s">
+        <v>53</v>
+      </c>
       <c r="O188" s="37" t="s">
         <v>464</v>
       </c>

</xml_diff>

<commit_message>
Update per id 452
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#ENTERXX/it.entersrl/it.entersrl.extralab/4.15.4.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#ENTERXX/it.entersrl/it.entersrl.extralab/4.15.4.0/report-checklist.xlsx
@@ -2204,13 +2204,13 @@
 </t>
   </si>
   <si>
-    <t>2026-03-12T14:51:45.7604111Z</t>
-  </si>
-  <si>
-    <t>053eaf6401bf3a299a6309a88563db05</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.adfc6ad043d682056f61756ce4dd65d9ba8a5023f67f0f6567153200ae19bcf6.b03ccc5093^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>2026-03-30T10:52:58.2197094Z</t>
+  </si>
+  <si>
+    <t>e6778b27ce72338d32dc44189e1e1526</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.adfc6ad043d682056f61756ce4dd65d9ba8a5023f67f0f6567153200ae19bcf6.d607263666^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_VPS_CT30</t>
@@ -3406,7 +3406,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -3517,6 +3517,9 @@
       <alignment horizontal="center" readingOrder="1" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="22" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="1" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="22" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="1" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
@@ -12381,7 +12384,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="168" ht="10.5" customHeight="1">
+    <row r="168">
       <c r="A168" s="33">
         <v>452.0</v>
       </c>
@@ -12398,15 +12401,15 @@
         <v>413</v>
       </c>
       <c r="F168" s="42">
-        <v>46093.0</v>
-      </c>
-      <c r="G168" s="42" t="s">
+        <v>46111.0</v>
+      </c>
+      <c r="G168" s="37" t="s">
         <v>414</v>
       </c>
-      <c r="H168" s="42" t="s">
+      <c r="H168" s="37" t="s">
         <v>415</v>
       </c>
-      <c r="I168" s="43" t="s">
+      <c r="I168" s="44" t="s">
         <v>416</v>
       </c>
       <c r="J168" s="38" t="s">
@@ -18350,42 +18353,42 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="45" t="s">
         <v>579</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="45" t="s">
         <v>580</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
-      <c r="A3" s="44" t="s">
+      <c r="A3" s="45" t="s">
         <v>581</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
-      <c r="A4" s="44" t="s">
+      <c r="A4" s="45" t="s">
         <v>582</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
-      <c r="A5" s="44" t="s">
+      <c r="A5" s="45" t="s">
         <v>583</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
-      <c r="A6" s="44" t="s">
+      <c r="A6" s="45" t="s">
         <v>584</v>
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1">
-      <c r="A7" s="44" t="s">
+      <c r="A7" s="45" t="s">
         <v>585</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
-      <c r="A8" s="44" t="s">
+      <c r="A8" s="45" t="s">
         <v>367</v>
       </c>
     </row>
@@ -19406,218 +19409,218 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="46" t="s">
         <v>586</v>
       </c>
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="47" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="46" t="s">
+      <c r="C1" s="47" t="s">
         <v>587</v>
       </c>
-      <c r="D1" s="46" t="s">
+      <c r="D1" s="47" t="s">
         <v>588</v>
       </c>
-      <c r="F1" s="47" t="s">
+      <c r="F1" s="48" t="s">
         <v>589</v>
       </c>
-      <c r="G1" s="48" t="s">
+      <c r="G1" s="49" t="s">
         <v>590</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
-      <c r="A2" s="49" t="s">
+      <c r="A2" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="B2" s="49" t="s">
+      <c r="B2" s="50" t="s">
         <v>591</v>
       </c>
-      <c r="C2" s="50" t="s">
+      <c r="C2" s="51" t="s">
         <v>592</v>
       </c>
-      <c r="D2" s="50" t="s">
+      <c r="D2" s="51" t="s">
         <v>593</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
-      <c r="A3" s="49" t="s">
+      <c r="A3" s="50" t="s">
         <v>63</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="B3" s="50" t="s">
         <v>591</v>
       </c>
-      <c r="C3" s="50" t="s">
+      <c r="C3" s="51" t="s">
         <v>594</v>
       </c>
-      <c r="D3" s="50" t="s">
+      <c r="D3" s="51" t="s">
         <v>595</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
-      <c r="A4" s="49" t="s">
+      <c r="A4" s="50" t="s">
         <v>69</v>
       </c>
-      <c r="B4" s="49" t="s">
+      <c r="B4" s="50" t="s">
         <v>591</v>
       </c>
-      <c r="C4" s="50" t="s">
+      <c r="C4" s="51" t="s">
         <v>596</v>
       </c>
-      <c r="D4" s="51" t="s">
+      <c r="D4" s="52" t="s">
         <v>597</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
-      <c r="A5" s="49" t="s">
+      <c r="A5" s="50" t="s">
         <v>75</v>
       </c>
-      <c r="B5" s="49" t="s">
+      <c r="B5" s="50" t="s">
         <v>591</v>
       </c>
-      <c r="C5" s="50" t="s">
+      <c r="C5" s="51" t="s">
         <v>598</v>
       </c>
-      <c r="D5" s="50" t="s">
+      <c r="D5" s="51" t="s">
         <v>599</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
-      <c r="A6" s="49" t="s">
+      <c r="A6" s="50" t="s">
         <v>78</v>
       </c>
-      <c r="B6" s="49" t="s">
+      <c r="B6" s="50" t="s">
         <v>591</v>
       </c>
-      <c r="C6" s="50" t="s">
+      <c r="C6" s="51" t="s">
         <v>600</v>
       </c>
-      <c r="D6" s="51" t="s">
+      <c r="D6" s="52" t="s">
         <v>601</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="49" t="s">
+      <c r="A7" s="50" t="s">
         <v>81</v>
       </c>
-      <c r="B7" s="49" t="s">
+      <c r="B7" s="50" t="s">
         <v>591</v>
       </c>
-      <c r="C7" s="50" t="s">
+      <c r="C7" s="51" t="s">
         <v>602</v>
       </c>
-      <c r="D7" s="51" t="s">
+      <c r="D7" s="52" t="s">
         <v>603</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="49" t="s">
+      <c r="A8" s="50" t="s">
         <v>72</v>
       </c>
-      <c r="B8" s="49" t="s">
+      <c r="B8" s="50" t="s">
         <v>591</v>
       </c>
-      <c r="C8" s="50" t="s">
+      <c r="C8" s="51" t="s">
         <v>604</v>
       </c>
-      <c r="D8" s="51" t="s">
+      <c r="D8" s="52" t="s">
         <v>605</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="49" t="s">
+      <c r="A9" s="50" t="s">
         <v>66</v>
       </c>
-      <c r="B9" s="49" t="s">
+      <c r="B9" s="50" t="s">
         <v>591</v>
       </c>
-      <c r="C9" s="50" t="s">
+      <c r="C9" s="51" t="s">
         <v>606</v>
       </c>
-      <c r="D9" s="51" t="s">
+      <c r="D9" s="52" t="s">
         <v>607</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="49" t="s">
+      <c r="A10" s="50" t="s">
         <v>608</v>
       </c>
-      <c r="B10" s="49" t="s">
+      <c r="B10" s="50" t="s">
         <v>591</v>
       </c>
-      <c r="C10" s="51" t="s">
+      <c r="C10" s="52" t="s">
         <v>609</v>
       </c>
-      <c r="D10" s="50" t="s">
+      <c r="D10" s="51" t="s">
         <v>610</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
-      <c r="A11" s="49" t="s">
+      <c r="A11" s="50" t="s">
         <v>371</v>
       </c>
-      <c r="B11" s="49" t="s">
+      <c r="B11" s="50" t="s">
         <v>591</v>
       </c>
-      <c r="C11" s="50" t="s">
+      <c r="C11" s="51" t="s">
         <v>611</v>
       </c>
-      <c r="D11" s="51" t="s">
+      <c r="D11" s="52" t="s">
         <v>612</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
-      <c r="A12" s="49" t="s">
+      <c r="A12" s="50" t="s">
         <v>475</v>
       </c>
-      <c r="B12" s="49" t="s">
+      <c r="B12" s="50" t="s">
         <v>591</v>
       </c>
-      <c r="C12" s="50" t="s">
+      <c r="C12" s="51" t="s">
         <v>613</v>
       </c>
-      <c r="D12" s="51" t="s">
+      <c r="D12" s="52" t="s">
         <v>614</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1">
-      <c r="A13" s="49" t="s">
+      <c r="A13" s="50" t="s">
         <v>499</v>
       </c>
-      <c r="B13" s="49" t="s">
+      <c r="B13" s="50" t="s">
         <v>591</v>
       </c>
-      <c r="C13" s="50" t="s">
+      <c r="C13" s="51" t="s">
         <v>615</v>
       </c>
-      <c r="D13" s="51" t="s">
+      <c r="D13" s="52" t="s">
         <v>616</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
-      <c r="A14" s="49" t="s">
+      <c r="A14" s="50" t="s">
         <v>529</v>
       </c>
-      <c r="B14" s="49" t="s">
+      <c r="B14" s="50" t="s">
         <v>591</v>
       </c>
-      <c r="C14" s="50" t="s">
+      <c r="C14" s="51" t="s">
         <v>617</v>
       </c>
-      <c r="D14" s="51" t="s">
+      <c r="D14" s="52" t="s">
         <v>618</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
-      <c r="A15" s="49" t="s">
+      <c r="A15" s="50" t="s">
         <v>559</v>
       </c>
-      <c r="B15" s="49" t="s">
+      <c r="B15" s="50" t="s">
         <v>591</v>
       </c>
-      <c r="C15" s="50">
+      <c r="C15" s="51">
         <v>521.0</v>
       </c>
-      <c r="D15" s="51" t="s">
+      <c r="D15" s="52" t="s">
         <v>619</v>
       </c>
     </row>
@@ -22598,26 +22601,26 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="53" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="52" t="s">
+      <c r="B1" s="53" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="53" t="s">
         <v>620</v>
       </c>
-      <c r="B2" s="52" t="s">
+      <c r="B2" s="53" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="53" t="s">
         <v>621</v>
       </c>
-      <c r="B3" s="52" t="s">
+      <c r="B3" s="53" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update traceid, workflowid e timespan test 4
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#ENTERXX/it.entersrl/it.entersrl.extralab/4.15.4.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#ENTERXX/it.entersrl/it.entersrl.extralab/4.15.4.0/report-checklist.xlsx
@@ -272,13 +272,13 @@
 </t>
   </si>
   <si>
-    <t>2026-03-30T10:04:51.0057722Z</t>
-  </si>
-  <si>
-    <t>1468ea0370385308add983fd42688fbf</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.c5deffffa6592522256b3f8a7279732f6069a3748f41f7c9f11ff0d9769302fa.bd762684d9^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>2026-03-30T13:44:29.5025161Z</t>
+  </si>
+  <si>
+    <t>0497e3396c00e52dde33833e1a0e60cf</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.80.3.1.4.4.c5deffffa6592522256b3f8a7279732f6069a3748f41f7c9f11ff0d9769302fa.cd6a0dfacf^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>SI</t>

</xml_diff>